<commit_message>
chore(data): batch update intraday meta_faturamento - 08:47:56
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -6793,7 +6793,7 @@
         <v>2621</v>
       </c>
       <c r="C578" t="n">
-        <v>43329</v>
+        <v>46662</v>
       </c>
     </row>
     <row r="579">
@@ -6804,7 +6804,7 @@
         <v>2737</v>
       </c>
       <c r="C579" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="580">
@@ -6815,7 +6815,7 @@
         <v>2090</v>
       </c>
       <c r="C580" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="581">
@@ -6826,7 +6826,7 @@
         <v>2310</v>
       </c>
       <c r="C581" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="582">
@@ -6837,7 +6837,7 @@
         <v>27</v>
       </c>
       <c r="C582" t="n">
-        <v>61893</v>
+        <v>66654</v>
       </c>
     </row>
     <row r="583">
@@ -6848,7 +6848,7 @@
         <v>522</v>
       </c>
       <c r="C583" t="n">
-        <v>123799</v>
+        <v>133322</v>
       </c>
     </row>
     <row r="584">
@@ -6859,7 +6859,7 @@
         <v>2676</v>
       </c>
       <c r="C584" t="n">
-        <v>38961</v>
+        <v>41958</v>
       </c>
     </row>
     <row r="585">
@@ -6870,7 +6870,7 @@
         <v>1380</v>
       </c>
       <c r="C585" t="n">
-        <v>61893</v>
+        <v>66654</v>
       </c>
     </row>
     <row r="586">
@@ -6881,7 +6881,7 @@
         <v>2069</v>
       </c>
       <c r="C586" t="n">
-        <v>111423</v>
+        <v>119994</v>
       </c>
     </row>
     <row r="587">
@@ -6892,7 +6892,7 @@
         <v>2734</v>
       </c>
       <c r="C587" t="n">
-        <v>34086</v>
+        <v>36708</v>
       </c>
     </row>
     <row r="588">
@@ -6903,7 +6903,7 @@
         <v>1137</v>
       </c>
       <c r="C588" t="n">
-        <v>383799</v>
+        <v>413322</v>
       </c>
     </row>
     <row r="589">
@@ -6914,7 +6914,7 @@
         <v>631</v>
       </c>
       <c r="C589" t="n">
-        <v>204282</v>
+        <v>219996</v>
       </c>
     </row>
     <row r="590">
@@ -6925,7 +6925,7 @@
         <v>2081</v>
       </c>
       <c r="C590" t="n">
-        <v>83564</v>
+        <v>89992</v>
       </c>
     </row>
     <row r="591">
@@ -6936,7 +6936,7 @@
         <v>2819</v>
       </c>
       <c r="C591" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="592">
@@ -6947,7 +6947,7 @@
         <v>2742</v>
       </c>
       <c r="C592" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="593">
@@ -6969,7 +6969,7 @@
         <v>1499</v>
       </c>
       <c r="C594" t="n">
-        <v>74282</v>
+        <v>79996</v>
       </c>
     </row>
     <row r="595">
@@ -6980,7 +6980,7 @@
         <v>2442</v>
       </c>
       <c r="C595" t="n">
-        <v>48282</v>
+        <v>51996</v>
       </c>
     </row>
     <row r="596">
@@ -6991,7 +6991,7 @@
         <v>772</v>
       </c>
       <c r="C596" t="n">
-        <v>217893</v>
+        <v>234654</v>
       </c>
     </row>
     <row r="597">
@@ -7002,7 +7002,7 @@
         <v>2728</v>
       </c>
       <c r="C597" t="n">
-        <v>99047.67999999999</v>
+        <v>106666.72</v>
       </c>
     </row>
     <row r="598">
@@ -7013,7 +7013,7 @@
         <v>1956</v>
       </c>
       <c r="C598" t="n">
-        <v>156297.3</v>
+        <v>168320.16</v>
       </c>
     </row>
     <row r="599">
@@ -7024,7 +7024,7 @@
         <v>2496</v>
       </c>
       <c r="C599" t="n">
-        <v>86658</v>
+        <v>93324</v>
       </c>
     </row>
     <row r="600">
@@ -7035,7 +7035,7 @@
         <v>2261</v>
       </c>
       <c r="C600" t="n">
-        <v>92846</v>
+        <v>99988</v>
       </c>
     </row>
     <row r="601">
@@ -7046,7 +7046,7 @@
         <v>2794</v>
       </c>
       <c r="C601" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="602">
@@ -7057,7 +7057,7 @@
         <v>2769</v>
       </c>
       <c r="C602" t="n">
-        <v>0.68</v>
+        <v>0.72</v>
       </c>
     </row>
     <row r="603">
@@ -7068,7 +7068,7 @@
         <v>2804</v>
       </c>
       <c r="C603" t="n">
-        <v>58799</v>
+        <v>63322</v>
       </c>
     </row>
     <row r="604">
@@ -7079,7 +7079,7 @@
         <v>2714</v>
       </c>
       <c r="C604" t="n">
-        <v>210470</v>
+        <v>226660</v>
       </c>
     </row>
     <row r="605">
@@ -7090,7 +7090,7 @@
         <v>2375</v>
       </c>
       <c r="C605" t="n">
-        <v>204282</v>
+        <v>219996</v>
       </c>
     </row>
     <row r="606">
@@ -7101,7 +7101,7 @@
         <v>1539</v>
       </c>
       <c r="C606" t="n">
-        <v>105235</v>
+        <v>113330</v>
       </c>
     </row>
     <row r="607">
@@ -7112,7 +7112,7 @@
         <v>2817</v>
       </c>
       <c r="C607" t="n">
-        <v>37141</v>
+        <v>39998</v>
       </c>
     </row>
     <row r="608">
@@ -7123,7 +7123,7 @@
         <v>2784</v>
       </c>
       <c r="C608" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="609">
@@ -7134,7 +7134,7 @@
         <v>2785</v>
       </c>
       <c r="C609" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="610">
@@ -7145,7 +7145,7 @@
         <v>2761</v>
       </c>
       <c r="C610" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="611">
@@ -7156,7 +7156,7 @@
         <v>2721</v>
       </c>
       <c r="C611" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="612">
@@ -7167,7 +7167,7 @@
         <v>2501</v>
       </c>
       <c r="C612" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="613">
@@ -7178,7 +7178,7 @@
         <v>1007</v>
       </c>
       <c r="C613" t="n">
-        <v>117611</v>
+        <v>126658</v>
       </c>
     </row>
     <row r="614">
@@ -7189,7 +7189,7 @@
         <v>1278</v>
       </c>
       <c r="C614" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="615">
@@ -7211,7 +7211,7 @@
         <v>2689</v>
       </c>
       <c r="C616" t="n">
-        <v>38961</v>
+        <v>41958</v>
       </c>
     </row>
     <row r="617">
@@ -7222,7 +7222,7 @@
         <v>20</v>
       </c>
       <c r="C617" t="n">
-        <v>241423</v>
+        <v>259994</v>
       </c>
     </row>
     <row r="618">
@@ -7233,7 +7233,7 @@
         <v>580</v>
       </c>
       <c r="C618" t="n">
-        <v>83564</v>
+        <v>89992</v>
       </c>
     </row>
     <row r="619">
@@ -7244,7 +7244,7 @@
         <v>2802</v>
       </c>
       <c r="C619" t="n">
-        <v>43836</v>
+        <v>47208</v>
       </c>
     </row>
     <row r="620">
@@ -7255,7 +7255,7 @@
         <v>1340</v>
       </c>
       <c r="C620" t="n">
-        <v>80470</v>
+        <v>86660</v>
       </c>
     </row>
     <row r="621">
@@ -7266,7 +7266,7 @@
         <v>358</v>
       </c>
       <c r="C621" t="n">
-        <v>219752</v>
+        <v>236656</v>
       </c>
     </row>
     <row r="622">
@@ -7277,7 +7277,7 @@
         <v>636</v>
       </c>
       <c r="C622" t="n">
-        <v>154752</v>
+        <v>166656</v>
       </c>
     </row>
     <row r="623">
@@ -7288,7 +7288,7 @@
         <v>1374</v>
       </c>
       <c r="C623" t="n">
-        <v>105235</v>
+        <v>113330</v>
       </c>
     </row>
     <row r="624">
@@ -7299,7 +7299,7 @@
         <v>2440</v>
       </c>
       <c r="C624" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="625">
@@ -7310,7 +7310,7 @@
         <v>429</v>
       </c>
       <c r="C625" t="n">
-        <v>241423</v>
+        <v>259994</v>
       </c>
     </row>
     <row r="626">
@@ -7321,7 +7321,7 @@
         <v>2015</v>
       </c>
       <c r="C626" t="n">
-        <v>219752</v>
+        <v>236656</v>
       </c>
     </row>
     <row r="627">
@@ -7332,7 +7332,7 @@
         <v>1259</v>
       </c>
       <c r="C627" t="n">
-        <v>61904.8</v>
+        <v>66666.7</v>
       </c>
     </row>
     <row r="628">
@@ -7343,7 +7343,7 @@
         <v>2346</v>
       </c>
       <c r="C628" t="n">
-        <v>68095.28</v>
+        <v>73333.37</v>
       </c>
     </row>
     <row r="629">
@@ -7354,7 +7354,7 @@
         <v>2431</v>
       </c>
       <c r="C629" t="n">
-        <v>116376</v>
+        <v>125328</v>
       </c>
     </row>
     <row r="630">
@@ -7365,7 +7365,7 @@
         <v>2792</v>
       </c>
       <c r="C630" t="n">
-        <v>72893.06</v>
+        <v>78500.21000000001</v>
       </c>
     </row>
     <row r="631">
@@ -7376,7 +7376,7 @@
         <v>2114</v>
       </c>
       <c r="C631" t="n">
-        <v>114753.11</v>
+        <v>123580.27</v>
       </c>
     </row>
     <row r="632">
@@ -7387,7 +7387,7 @@
         <v>2359</v>
       </c>
       <c r="C632" t="n">
-        <v>69615.25999999999</v>
+        <v>74970.27</v>
       </c>
     </row>
     <row r="633">
@@ -7398,7 +7398,7 @@
         <v>1142</v>
       </c>
       <c r="C633" t="n">
-        <v>265603</v>
+        <v>286034</v>
       </c>
     </row>
     <row r="634">
@@ -7409,7 +7409,7 @@
         <v>569</v>
       </c>
       <c r="C634" t="n">
-        <v>1772901</v>
+        <v>1909278</v>
       </c>
     </row>
     <row r="635">
@@ -7442,7 +7442,7 @@
         <v>2333</v>
       </c>
       <c r="C637" t="n">
-        <v>95550</v>
+        <v>102900</v>
       </c>
     </row>
     <row r="638">
@@ -7453,7 +7453,7 @@
         <v>2707</v>
       </c>
       <c r="C638" t="n">
-        <v>19840.56</v>
+        <v>21366.74</v>
       </c>
     </row>
     <row r="639">
@@ -7464,7 +7464,7 @@
         <v>2472</v>
       </c>
       <c r="C639" t="n">
-        <v>29869.12</v>
+        <v>32166.73</v>
       </c>
     </row>
     <row r="640">
@@ -7508,7 +7508,7 @@
         <v>2498</v>
       </c>
       <c r="C643" t="n">
-        <v>30966</v>
+        <v>33348</v>
       </c>
     </row>
     <row r="644">
@@ -7519,7 +7519,7 @@
         <v>2381</v>
       </c>
       <c r="C644" t="n">
-        <v>44239</v>
+        <v>47642</v>
       </c>
     </row>
     <row r="645">
@@ -7530,7 +7530,7 @@
         <v>2273</v>
       </c>
       <c r="C645" t="n">
-        <v>118261</v>
+        <v>127358</v>
       </c>
     </row>
     <row r="646">
@@ -7541,7 +7541,7 @@
         <v>2647</v>
       </c>
       <c r="C646" t="n">
-        <v>87841</v>
+        <v>94598</v>
       </c>
     </row>
     <row r="647">
@@ -7552,7 +7552,7 @@
         <v>2492</v>
       </c>
       <c r="C647" t="n">
-        <v>87841</v>
+        <v>94598</v>
       </c>
     </row>
     <row r="648">
@@ -7563,7 +7563,7 @@
         <v>2631</v>
       </c>
       <c r="C648" t="n">
-        <v>15197.68</v>
+        <v>16366.72</v>
       </c>
     </row>
     <row r="649">
@@ -7574,7 +7574,7 @@
         <v>2682</v>
       </c>
       <c r="C649" t="n">
-        <v>185714.4</v>
+        <v>200000.1</v>
       </c>
     </row>
     <row r="650">
@@ -7585,7 +7585,7 @@
         <v>1075</v>
       </c>
       <c r="C650" t="n">
-        <v>280423</v>
+        <v>301994</v>
       </c>
     </row>
     <row r="651">
@@ -7596,7 +7596,7 @@
         <v>2810</v>
       </c>
       <c r="C651" t="n">
-        <v>86658</v>
+        <v>93324</v>
       </c>
     </row>
     <row r="652">
@@ -7607,7 +7607,7 @@
         <v>2547</v>
       </c>
       <c r="C652" t="n">
-        <v>25467</v>
+        <v>27426</v>
       </c>
     </row>
     <row r="653">
@@ -7618,7 +7618,7 @@
         <v>2627</v>
       </c>
       <c r="C653" t="n">
-        <v>15093</v>
+        <v>16254</v>
       </c>
     </row>
     <row r="654">
@@ -7640,7 +7640,7 @@
         <v>2562</v>
       </c>
       <c r="C655" t="n">
-        <v>9802</v>
+        <v>10556</v>
       </c>
     </row>
     <row r="656">
@@ -7651,7 +7651,7 @@
         <v>1658</v>
       </c>
       <c r="C656" t="n">
-        <v>84188</v>
+        <v>90664</v>
       </c>
     </row>
     <row r="657">
@@ -7662,7 +7662,7 @@
         <v>1996</v>
       </c>
       <c r="C657" t="n">
-        <v>217126</v>
+        <v>233828</v>
       </c>
     </row>
     <row r="658">
@@ -7673,7 +7673,7 @@
         <v>2674</v>
       </c>
       <c r="C658" t="n">
-        <v>160940</v>
+        <v>173320</v>
       </c>
     </row>
     <row r="659">
@@ -7684,7 +7684,7 @@
         <v>2163</v>
       </c>
       <c r="C659" t="n">
-        <v>86658</v>
+        <v>93324</v>
       </c>
     </row>
     <row r="660">
@@ -7706,7 +7706,7 @@
         <v>1834</v>
       </c>
       <c r="C661" t="n">
-        <v>72423</v>
+        <v>77994</v>
       </c>
     </row>
     <row r="662">
@@ -7717,7 +7717,7 @@
         <v>2109</v>
       </c>
       <c r="C662" t="n">
-        <v>57880.96</v>
+        <v>62333.34</v>
       </c>
     </row>
     <row r="663">
@@ -7761,7 +7761,7 @@
         <v>630</v>
       </c>
       <c r="C666" t="n">
-        <v>16718</v>
+        <v>18004</v>
       </c>
     </row>
     <row r="667">
@@ -7772,7 +7772,7 @@
         <v>2197</v>
       </c>
       <c r="C667" t="n">
-        <v>123799</v>
+        <v>133322</v>
       </c>
     </row>
     <row r="668">
@@ -7794,7 +7794,7 @@
         <v>1983</v>
       </c>
       <c r="C669" t="n">
-        <v>358930</v>
+        <v>386540</v>
       </c>
     </row>
     <row r="670">
@@ -7805,7 +7805,7 @@
         <v>941</v>
       </c>
       <c r="C670" t="n">
-        <v>219005.45</v>
+        <v>235852.01</v>
       </c>
     </row>
     <row r="671">
@@ -7827,7 +7827,7 @@
         <v>2556</v>
       </c>
       <c r="C672" t="n">
-        <v>22347</v>
+        <v>24066</v>
       </c>
     </row>
     <row r="673">
@@ -7849,7 +7849,7 @@
         <v>1993</v>
       </c>
       <c r="C674" t="n">
-        <v>215358</v>
+        <v>231924</v>
       </c>
     </row>
     <row r="675">
@@ -7860,7 +7860,7 @@
         <v>949</v>
       </c>
       <c r="C675" t="n">
-        <v>60762</v>
+        <v>65436</v>
       </c>
     </row>
     <row r="676">
@@ -7871,7 +7871,7 @@
         <v>1298</v>
       </c>
       <c r="C676" t="n">
-        <v>695344</v>
+        <v>748832</v>
       </c>
     </row>
     <row r="677">
@@ -7882,7 +7882,7 @@
         <v>2729</v>
       </c>
       <c r="C677" t="n">
-        <v>30940</v>
+        <v>33320</v>
       </c>
     </row>
     <row r="678">
@@ -7893,7 +7893,7 @@
         <v>1873</v>
       </c>
       <c r="C678" t="n">
-        <v>197470</v>
+        <v>212660</v>
       </c>
     </row>
     <row r="679">
@@ -7904,7 +7904,7 @@
         <v>1466</v>
       </c>
       <c r="C679" t="n">
-        <v>244517</v>
+        <v>263326</v>
       </c>
     </row>
     <row r="680">
@@ -7915,7 +7915,7 @@
         <v>2671</v>
       </c>
       <c r="C680" t="n">
-        <v>49517</v>
+        <v>53326</v>
       </c>
     </row>
     <row r="681">
@@ -7926,7 +7926,7 @@
         <v>2786</v>
       </c>
       <c r="C681" t="n">
-        <v>43329</v>
+        <v>46662</v>
       </c>
     </row>
     <row r="682">
@@ -7937,7 +7937,7 @@
         <v>2073</v>
       </c>
       <c r="C682" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="683">
@@ -7948,7 +7948,7 @@
         <v>2583</v>
       </c>
       <c r="C683" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="684">
@@ -7959,7 +7959,7 @@
         <v>2796</v>
       </c>
       <c r="C684" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="685">
@@ -7970,7 +7970,7 @@
         <v>1384</v>
       </c>
       <c r="C685" t="n">
-        <v>278564</v>
+        <v>299992</v>
       </c>
     </row>
     <row r="686">
@@ -7981,7 +7981,7 @@
         <v>132</v>
       </c>
       <c r="C686" t="n">
-        <v>464282</v>
+        <v>499996</v>
       </c>
     </row>
     <row r="687">
@@ -7992,7 +7992,7 @@
         <v>1518</v>
       </c>
       <c r="C687" t="n">
-        <v>216658</v>
+        <v>233324</v>
       </c>
     </row>
     <row r="688">
@@ -8003,7 +8003,7 @@
         <v>438</v>
       </c>
       <c r="C688" t="n">
-        <v>95940</v>
+        <v>103320</v>
       </c>
     </row>
     <row r="689">
@@ -8014,7 +8014,7 @@
         <v>2716</v>
       </c>
       <c r="C689" t="n">
-        <v>53573</v>
+        <v>57694</v>
       </c>
     </row>
     <row r="690">
@@ -8025,7 +8025,7 @@
         <v>14</v>
       </c>
       <c r="C690" t="n">
-        <v>269282</v>
+        <v>289996</v>
       </c>
     </row>
     <row r="691">
@@ -8036,7 +8036,7 @@
         <v>535</v>
       </c>
       <c r="C691" t="n">
-        <v>235235</v>
+        <v>253330</v>
       </c>
     </row>
     <row r="692">
@@ -8047,7 +8047,7 @@
         <v>2795</v>
       </c>
       <c r="C692" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="693">
@@ -8058,7 +8058,7 @@
         <v>1456</v>
       </c>
       <c r="C693" t="n">
-        <v>476840</v>
+        <v>513520</v>
       </c>
     </row>
     <row r="694">
@@ -8069,7 +8069,7 @@
         <v>2249</v>
       </c>
       <c r="C694" t="n">
-        <v>120913</v>
+        <v>130214</v>
       </c>
     </row>
     <row r="695">
@@ -8080,7 +8080,7 @@
         <v>2394</v>
       </c>
       <c r="C695" t="n">
-        <v>95368</v>
+        <v>102704</v>
       </c>
     </row>
     <row r="696">
@@ -8091,7 +8091,7 @@
         <v>2507</v>
       </c>
       <c r="C696" t="n">
-        <v>56834.98</v>
+        <v>61206.9</v>
       </c>
     </row>
     <row r="697">
@@ -8102,7 +8102,7 @@
         <v>2697</v>
       </c>
       <c r="C697" t="n">
-        <v>119198.55</v>
+        <v>128367.66</v>
       </c>
     </row>
     <row r="698">
@@ -8113,7 +8113,7 @@
         <v>2698</v>
       </c>
       <c r="C698" t="n">
-        <v>75631.03</v>
+        <v>81448.78999999999</v>
       </c>
     </row>
     <row r="699">
@@ -8124,7 +8124,7 @@
         <v>2510</v>
       </c>
       <c r="C699" t="n">
-        <v>343720</v>
+        <v>370160</v>
       </c>
     </row>
     <row r="700">
@@ -8135,7 +8135,7 @@
         <v>2613</v>
       </c>
       <c r="C700" t="n">
-        <v>110916</v>
+        <v>119448</v>
       </c>
     </row>
     <row r="701">
@@ -8146,7 +8146,7 @@
         <v>2820</v>
       </c>
       <c r="C701" t="n">
-        <v>111428.64</v>
+        <v>120000.06</v>
       </c>
     </row>
     <row r="702">
@@ -8157,7 +8157,7 @@
         <v>2000</v>
       </c>
       <c r="C702" t="n">
-        <v>61285.76</v>
+        <v>66000.03999999999</v>
       </c>
     </row>
     <row r="703">
@@ -8168,7 +8168,7 @@
         <v>1871</v>
       </c>
       <c r="C703" t="n">
-        <v>109421</v>
+        <v>117838</v>
       </c>
     </row>
     <row r="704">
@@ -8201,7 +8201,7 @@
         <v>2145</v>
       </c>
       <c r="C706" t="n">
-        <v>80132</v>
+        <v>86296</v>
       </c>
     </row>
     <row r="707">
@@ -8212,7 +8212,7 @@
         <v>2574</v>
       </c>
       <c r="C707" t="n">
-        <v>80132</v>
+        <v>86296</v>
       </c>
     </row>
     <row r="708">
@@ -8223,7 +8223,7 @@
         <v>2411</v>
       </c>
       <c r="C708" t="n">
-        <v>87841</v>
+        <v>94598</v>
       </c>
     </row>
     <row r="709">
@@ -8234,7 +8234,7 @@
         <v>2692</v>
       </c>
       <c r="C709" t="n">
-        <v>46428.64</v>
+        <v>50000.06</v>
       </c>
     </row>
     <row r="710">
@@ -8245,7 +8245,7 @@
         <v>945</v>
       </c>
       <c r="C710" t="n">
-        <v>175397.63</v>
+        <v>188889.74</v>
       </c>
     </row>
     <row r="711">
@@ -8267,7 +8267,7 @@
         <v>664</v>
       </c>
       <c r="C712" t="n">
-        <v>165893</v>
+        <v>178654</v>
       </c>
     </row>
     <row r="713">
@@ -8289,7 +8289,7 @@
         <v>947</v>
       </c>
       <c r="C714" t="n">
-        <v>269001.37</v>
+        <v>289693.78</v>
       </c>
     </row>
     <row r="715">
@@ -8311,7 +8311,7 @@
         <v>2279</v>
       </c>
       <c r="C716" t="n">
-        <v>143572</v>
+        <v>154616</v>
       </c>
     </row>
     <row r="717">
@@ -8322,7 +8322,7 @@
         <v>58</v>
       </c>
       <c r="C717" t="n">
-        <v>143572</v>
+        <v>154616</v>
       </c>
     </row>
     <row r="718">
@@ -8333,7 +8333,7 @@
         <v>2648</v>
       </c>
       <c r="C718" t="n">
-        <v>89752</v>
+        <v>96656</v>
       </c>
     </row>
     <row r="719">
@@ -8355,7 +8355,7 @@
         <v>2558</v>
       </c>
       <c r="C720" t="n">
-        <v>18603</v>
+        <v>20034</v>
       </c>
     </row>
     <row r="721">
@@ -8366,7 +8366,7 @@
         <v>2245</v>
       </c>
       <c r="C721" t="n">
-        <v>143572</v>
+        <v>154616</v>
       </c>
     </row>
     <row r="722">
@@ -8377,7 +8377,7 @@
         <v>1064</v>
       </c>
       <c r="C722" t="n">
-        <v>371033</v>
+        <v>399574</v>
       </c>
     </row>
     <row r="723">
@@ -8388,7 +8388,7 @@
         <v>2557</v>
       </c>
       <c r="C723" t="n">
-        <v>15951</v>
+        <v>17178</v>
       </c>
     </row>
     <row r="724">
@@ -8399,7 +8399,7 @@
         <v>360</v>
       </c>
       <c r="C724" t="n">
-        <v>309517</v>
+        <v>333326</v>
       </c>
     </row>
     <row r="725">
@@ -8410,7 +8410,7 @@
         <v>2767</v>
       </c>
       <c r="C725" t="n">
-        <v>119431</v>
+        <v>128618</v>
       </c>
     </row>
     <row r="726">
@@ -8421,7 +8421,7 @@
         <v>781</v>
       </c>
       <c r="C726" t="n">
-        <v>80470</v>
+        <v>86660</v>
       </c>
     </row>
     <row r="727">
@@ -8432,7 +8432,7 @@
         <v>1020</v>
       </c>
       <c r="C727" t="n">
-        <v>52611</v>
+        <v>56658</v>
       </c>
     </row>
     <row r="728">
@@ -8454,7 +8454,7 @@
         <v>2258</v>
       </c>
       <c r="C729" t="n">
-        <v>49523.84</v>
+        <v>53333.36</v>
       </c>
     </row>
     <row r="730">
@@ -8465,7 +8465,7 @@
         <v>2744</v>
       </c>
       <c r="C730" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="731">
@@ -8476,7 +8476,7 @@
         <v>2758</v>
       </c>
       <c r="C731" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="732">
@@ -8487,7 +8487,7 @@
         <v>2772</v>
       </c>
       <c r="C732" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="733">
@@ -8498,7 +8498,7 @@
         <v>2797</v>
       </c>
       <c r="C733" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="734">
@@ -8509,7 +8509,7 @@
         <v>2815</v>
       </c>
       <c r="C734" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="735">
@@ -8520,7 +8520,7 @@
         <v>1869</v>
       </c>
       <c r="C735" t="n">
-        <v>141141</v>
+        <v>151998</v>
       </c>
     </row>
     <row r="736">
@@ -8531,7 +8531,7 @@
         <v>452</v>
       </c>
       <c r="C736" t="n">
-        <v>160940</v>
+        <v>173320</v>
       </c>
     </row>
     <row r="737">
@@ -8542,7 +8542,7 @@
         <v>2178</v>
       </c>
       <c r="C737" t="n">
-        <v>182611</v>
+        <v>196658</v>
       </c>
     </row>
     <row r="738">
@@ -8553,7 +8553,7 @@
         <v>1308</v>
       </c>
       <c r="C738" t="n">
-        <v>98606.62</v>
+        <v>106191.74</v>
       </c>
     </row>
     <row r="739">
@@ -8564,7 +8564,7 @@
         <v>2107</v>
       </c>
       <c r="C739" t="n">
-        <v>172621.09</v>
+        <v>185899.63</v>
       </c>
     </row>
     <row r="740">
@@ -8575,7 +8575,7 @@
         <v>2211</v>
       </c>
       <c r="C740" t="n">
-        <v>138548.86</v>
+        <v>149206.45</v>
       </c>
     </row>
     <row r="741">
@@ -8586,7 +8586,7 @@
         <v>2567</v>
       </c>
       <c r="C741" t="n">
-        <v>102180</v>
+        <v>110040</v>
       </c>
     </row>
     <row r="742">
@@ -8597,7 +8597,7 @@
         <v>2680</v>
       </c>
       <c r="C742" t="n">
-        <v>66906.81</v>
+        <v>72053.48</v>
       </c>
     </row>
     <row r="743">
@@ -8608,7 +8608,7 @@
         <v>2568</v>
       </c>
       <c r="C743" t="n">
-        <v>126542</v>
+        <v>136276</v>
       </c>
     </row>
     <row r="744">
@@ -8619,7 +8619,7 @@
         <v>2790</v>
       </c>
       <c r="C744" t="n">
-        <v>33428.64</v>
+        <v>36000.06</v>
       </c>
     </row>
     <row r="745">
@@ -8641,7 +8641,7 @@
         <v>2250</v>
       </c>
       <c r="C746" t="n">
-        <v>204841</v>
+        <v>220598</v>
       </c>
     </row>
     <row r="747">
@@ -8652,7 +8652,7 @@
         <v>2705</v>
       </c>
       <c r="C747" t="n">
-        <v>110916</v>
+        <v>119448</v>
       </c>
     </row>
     <row r="748">
@@ -8663,7 +8663,7 @@
         <v>2082</v>
       </c>
       <c r="C748" t="n">
-        <v>103116</v>
+        <v>111048</v>
       </c>
     </row>
     <row r="749">
@@ -8674,7 +8674,7 @@
         <v>2183</v>
       </c>
       <c r="C749" t="n">
-        <v>226551</v>
+        <v>243978</v>
       </c>
     </row>
     <row r="750">
@@ -8685,7 +8685,7 @@
         <v>2276</v>
       </c>
       <c r="C750" t="n">
-        <v>138697</v>
+        <v>149366</v>
       </c>
     </row>
     <row r="751">
@@ -8696,7 +8696,7 @@
         <v>477</v>
       </c>
       <c r="C751" t="n">
-        <v>160121</v>
+        <v>172438</v>
       </c>
     </row>
     <row r="752">
@@ -8707,7 +8707,7 @@
         <v>2691</v>
       </c>
       <c r="C752" t="n">
-        <v>83571.44</v>
+        <v>90000.00999999999</v>
       </c>
     </row>
     <row r="753">
@@ -8718,7 +8718,7 @@
         <v>1289</v>
       </c>
       <c r="C753" t="n">
-        <v>154752</v>
+        <v>166656</v>
       </c>
     </row>
     <row r="754">
@@ -8729,7 +8729,7 @@
         <v>1632</v>
       </c>
       <c r="C754" t="n">
-        <v>154752</v>
+        <v>166656</v>
       </c>
     </row>
     <row r="755">
@@ -8740,7 +8740,7 @@
         <v>2801</v>
       </c>
       <c r="C755" t="n">
-        <v>86658</v>
+        <v>93324</v>
       </c>
     </row>
     <row r="756">
@@ -8751,7 +8751,7 @@
         <v>451</v>
       </c>
       <c r="C756" t="n">
-        <v>154752</v>
+        <v>166656</v>
       </c>
     </row>
     <row r="757">
@@ -8762,7 +8762,7 @@
         <v>1102</v>
       </c>
       <c r="C757" t="n">
-        <v>143572</v>
+        <v>154616</v>
       </c>
     </row>
     <row r="758">
@@ -8773,7 +8773,7 @@
         <v>1465</v>
       </c>
       <c r="C758" t="n">
-        <v>222716</v>
+        <v>239848</v>
       </c>
     </row>
     <row r="759">
@@ -8784,7 +8784,7 @@
         <v>2649</v>
       </c>
       <c r="C759" t="n">
-        <v>18278</v>
+        <v>19684</v>
       </c>
     </row>
     <row r="760">
@@ -8795,7 +8795,7 @@
         <v>400</v>
       </c>
       <c r="C760" t="n">
-        <v>114517</v>
+        <v>123326</v>
       </c>
     </row>
     <row r="761">
@@ -8806,7 +8806,7 @@
         <v>2133</v>
       </c>
       <c r="C761" t="n">
-        <v>497705</v>
+        <v>535990</v>
       </c>
     </row>
     <row r="762">
@@ -8817,7 +8817,7 @@
         <v>767</v>
       </c>
       <c r="C762" t="n">
-        <v>111428.64</v>
+        <v>120000.06</v>
       </c>
     </row>
     <row r="763">
@@ -8828,7 +8828,7 @@
         <v>2516</v>
       </c>
       <c r="C763" t="n">
-        <v>68095.28</v>
+        <v>73333.37</v>
       </c>
     </row>
     <row r="764">
@@ -8839,7 +8839,7 @@
         <v>2722</v>
       </c>
       <c r="C764" t="n">
-        <v>24752</v>
+        <v>26656</v>
       </c>
     </row>
     <row r="765">
@@ -8850,7 +8850,7 @@
         <v>2566</v>
       </c>
       <c r="C765" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="766">
@@ -8861,7 +8861,7 @@
         <v>2635</v>
       </c>
       <c r="C766" t="n">
-        <v>80470</v>
+        <v>86660</v>
       </c>
     </row>
     <row r="767">
@@ -8872,7 +8872,7 @@
         <v>2726</v>
       </c>
       <c r="C767" t="n">
-        <v>92857.2</v>
+        <v>100000.05</v>
       </c>
     </row>
     <row r="768">
@@ -8883,7 +8883,7 @@
         <v>2730</v>
       </c>
       <c r="C768" t="n">
-        <v>55714.32</v>
+        <v>60000.03</v>
       </c>
     </row>
     <row r="769">
@@ -8894,7 +8894,7 @@
         <v>2765</v>
       </c>
       <c r="C769" t="n">
-        <v>58799</v>
+        <v>63322</v>
       </c>
     </row>
     <row r="770">
@@ -8905,7 +8905,7 @@
         <v>2735</v>
       </c>
       <c r="C770" t="n">
-        <v>74282</v>
+        <v>79996</v>
       </c>
     </row>
     <row r="771">
@@ -8916,7 +8916,7 @@
         <v>2816</v>
       </c>
       <c r="C771" t="n">
-        <v>30940</v>
+        <v>33320</v>
       </c>
     </row>
     <row r="772">
@@ -8927,7 +8927,7 @@
         <v>1881</v>
       </c>
       <c r="C772" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="773">
@@ -8938,7 +8938,7 @@
         <v>595</v>
       </c>
       <c r="C773" t="n">
-        <v>340470</v>
+        <v>366660</v>
       </c>
     </row>
     <row r="774">
@@ -8949,7 +8949,7 @@
         <v>925</v>
       </c>
       <c r="C774" t="n">
-        <v>48711</v>
+        <v>52458</v>
       </c>
     </row>
     <row r="775">
@@ -8960,7 +8960,7 @@
         <v>2582</v>
       </c>
       <c r="C775" t="n">
-        <v>53573</v>
+        <v>57694</v>
       </c>
     </row>
     <row r="776">
@@ -8971,7 +8971,7 @@
         <v>2637</v>
       </c>
       <c r="C776" t="n">
-        <v>38961</v>
+        <v>41958</v>
       </c>
     </row>
     <row r="777">
@@ -8982,7 +8982,7 @@
         <v>2448</v>
       </c>
       <c r="C777" t="n">
-        <v>43329</v>
+        <v>46662</v>
       </c>
     </row>
     <row r="778">
@@ -8993,7 +8993,7 @@
         <v>2452</v>
       </c>
       <c r="C778" t="n">
-        <v>40235</v>
+        <v>43330</v>
       </c>
     </row>
     <row r="779">
@@ -9004,7 +9004,7 @@
         <v>2362</v>
       </c>
       <c r="C779" t="n">
-        <v>43329</v>
+        <v>46662</v>
       </c>
     </row>
     <row r="780">
@@ -9015,7 +9015,7 @@
         <v>1277</v>
       </c>
       <c r="C780" t="n">
-        <v>136188</v>
+        <v>146664</v>
       </c>
     </row>
     <row r="781">
@@ -9026,7 +9026,7 @@
         <v>1327</v>
       </c>
       <c r="C781" t="n">
-        <v>30940</v>
+        <v>33320</v>
       </c>
     </row>
     <row r="782">
@@ -9037,7 +9037,7 @@
         <v>2599</v>
       </c>
       <c r="C782" t="n">
-        <v>117000</v>
+        <v>126000</v>
       </c>
     </row>
     <row r="783">
@@ -9048,7 +9048,7 @@
         <v>2402</v>
       </c>
       <c r="C783" t="n">
-        <v>403611</v>
+        <v>434658</v>
       </c>
     </row>
     <row r="784">
@@ -9059,7 +9059,7 @@
         <v>2085</v>
       </c>
       <c r="C784" t="n">
-        <v>81744</v>
+        <v>88032</v>
       </c>
     </row>
     <row r="785">
@@ -9081,7 +9081,7 @@
         <v>2341</v>
       </c>
       <c r="C786" t="n">
-        <v>87841</v>
+        <v>94598</v>
       </c>
     </row>
     <row r="787">
@@ -9092,7 +9092,7 @@
         <v>2667</v>
       </c>
       <c r="C787" t="n">
-        <v>22285.84</v>
+        <v>24000.11</v>
       </c>
     </row>
     <row r="788">
@@ -9103,7 +9103,7 @@
         <v>1372</v>
       </c>
       <c r="C788" t="n">
-        <v>179517</v>
+        <v>193326</v>
       </c>
     </row>
     <row r="789">
@@ -9114,7 +9114,7 @@
         <v>1653</v>
       </c>
       <c r="C789" t="n">
-        <v>207376</v>
+        <v>223328</v>
       </c>
     </row>
     <row r="790">
@@ -9125,7 +9125,7 @@
         <v>1324</v>
       </c>
       <c r="C790" t="n">
-        <v>173329</v>
+        <v>186662</v>
       </c>
     </row>
     <row r="791">
@@ -9136,7 +9136,7 @@
         <v>802</v>
       </c>
       <c r="C791" t="n">
-        <v>46423</v>
+        <v>49994</v>
       </c>
     </row>
     <row r="792">
@@ -9147,7 +9147,7 @@
         <v>2747</v>
       </c>
       <c r="C792" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="793">
@@ -9158,7 +9158,7 @@
         <v>2798</v>
       </c>
       <c r="C793" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="794">
@@ -9169,7 +9169,7 @@
         <v>33</v>
       </c>
       <c r="C794" t="n">
-        <v>240799</v>
+        <v>259322</v>
       </c>
     </row>
     <row r="795">
@@ -9180,7 +9180,7 @@
         <v>783</v>
       </c>
       <c r="C795" t="n">
-        <v>27846</v>
+        <v>29988</v>
       </c>
     </row>
     <row r="796">
@@ -9191,7 +9191,7 @@
         <v>2768</v>
       </c>
       <c r="C796" t="n">
-        <v>206684.91</v>
+        <v>222583.74</v>
       </c>
     </row>
     <row r="797">
@@ -9202,7 +9202,7 @@
         <v>2491</v>
       </c>
       <c r="C797" t="n">
-        <v>67741.53999999999</v>
+        <v>72952.42</v>
       </c>
     </row>
     <row r="798">
@@ -9213,7 +9213,7 @@
         <v>2606</v>
       </c>
       <c r="C798" t="n">
-        <v>146458</v>
+        <v>157724</v>
       </c>
     </row>
     <row r="799">
@@ -9224,7 +9224,7 @@
         <v>2799</v>
       </c>
       <c r="C799" t="n">
-        <v>73042.89999999999</v>
+        <v>78661.58</v>
       </c>
     </row>
     <row r="800">
@@ -9235,7 +9235,7 @@
         <v>2571</v>
       </c>
       <c r="C800" t="n">
-        <v>96773.62</v>
+        <v>104217.74</v>
       </c>
     </row>
     <row r="801">
@@ -9246,7 +9246,7 @@
         <v>2696</v>
       </c>
       <c r="C801" t="n">
-        <v>151657.6</v>
+        <v>163323.56</v>
       </c>
     </row>
     <row r="802">
@@ -9257,7 +9257,7 @@
         <v>1907</v>
       </c>
       <c r="C802" t="n">
-        <v>229658</v>
+        <v>247324</v>
       </c>
     </row>
     <row r="803">
@@ -9268,7 +9268,7 @@
         <v>2392</v>
       </c>
       <c r="C803" t="n">
-        <v>103116</v>
+        <v>111048</v>
       </c>
     </row>
     <row r="804">
@@ -9279,7 +9279,7 @@
         <v>2706</v>
       </c>
       <c r="C804" t="n">
-        <v>10554.88</v>
+        <v>11366.77</v>
       </c>
     </row>
     <row r="805">
@@ -9290,7 +9290,7 @@
         <v>2657</v>
       </c>
       <c r="C805" t="n">
-        <v>49214.4</v>
+        <v>53000.1</v>
       </c>
     </row>
     <row r="806">
@@ -9312,7 +9312,7 @@
         <v>2695</v>
       </c>
       <c r="C807" t="n">
-        <v>26611</v>
+        <v>28658</v>
       </c>
     </row>
     <row r="808">
@@ -9323,7 +9323,7 @@
         <v>2700</v>
       </c>
       <c r="C808" t="n">
-        <v>33618</v>
+        <v>36204</v>
       </c>
     </row>
     <row r="809">
@@ -9334,7 +9334,7 @@
         <v>1800</v>
       </c>
       <c r="C809" t="n">
-        <v>15600</v>
+        <v>16800</v>
       </c>
     </row>
     <row r="810">
@@ -9345,7 +9345,7 @@
         <v>2541</v>
       </c>
       <c r="C810" t="n">
-        <v>130988</v>
+        <v>141064</v>
       </c>
     </row>
     <row r="811">
@@ -9356,7 +9356,7 @@
         <v>2365</v>
       </c>
       <c r="C811" t="n">
-        <v>49309</v>
+        <v>53102</v>
       </c>
     </row>
     <row r="812">
@@ -9367,7 +9367,7 @@
         <v>1890</v>
       </c>
       <c r="C812" t="n">
-        <v>175237.42</v>
+        <v>188717.2</v>
       </c>
     </row>
     <row r="813">
@@ -9389,7 +9389,7 @@
         <v>1299</v>
       </c>
       <c r="C814" t="n">
-        <v>322114</v>
+        <v>346892</v>
       </c>
     </row>
     <row r="815">
@@ -9422,7 +9422,7 @@
         <v>1937</v>
       </c>
       <c r="C817" t="n">
-        <v>160680</v>
+        <v>173040</v>
       </c>
     </row>
     <row r="818">
@@ -9433,7 +9433,7 @@
         <v>610</v>
       </c>
       <c r="C818" t="n">
-        <v>507819</v>
+        <v>546882</v>
       </c>
     </row>
     <row r="819">
@@ -9444,7 +9444,7 @@
         <v>131</v>
       </c>
       <c r="C819" t="n">
-        <v>253188</v>
+        <v>272664</v>
       </c>
     </row>
     <row r="820">
@@ -9455,7 +9455,7 @@
         <v>2789</v>
       </c>
       <c r="C820" t="n">
-        <v>105235</v>
+        <v>113330</v>
       </c>
     </row>
     <row r="821">
@@ -9488,7 +9488,7 @@
         <v>629</v>
       </c>
       <c r="C823" t="n">
-        <v>271752</v>
+        <v>292656</v>
       </c>
     </row>
     <row r="824">
@@ -9521,7 +9521,7 @@
         <v>285</v>
       </c>
       <c r="C826" t="n">
-        <v>358930</v>
+        <v>386540</v>
       </c>
     </row>
     <row r="827">
@@ -9532,7 +9532,7 @@
         <v>2643</v>
       </c>
       <c r="C827" t="n">
-        <v>18278</v>
+        <v>19684</v>
       </c>
     </row>
     <row r="828">
@@ -9543,7 +9543,7 @@
         <v>2421</v>
       </c>
       <c r="C828" t="n">
-        <v>35282</v>
+        <v>37996</v>
       </c>
     </row>
     <row r="829">
@@ -9554,7 +9554,7 @@
         <v>571</v>
       </c>
       <c r="C829" t="n">
-        <v>335738</v>
+        <v>361564</v>
       </c>
     </row>
     <row r="830">
@@ -9565,7 +9565,7 @@
         <v>2686</v>
       </c>
       <c r="C830" t="n">
-        <v>80476.24000000001</v>
+        <v>86666.71000000001</v>
       </c>
     </row>
     <row r="831">
@@ -9576,7 +9576,7 @@
         <v>2494</v>
       </c>
       <c r="C831" t="n">
-        <v>80470</v>
+        <v>86660</v>
       </c>
     </row>
     <row r="832">
@@ -9587,7 +9587,7 @@
         <v>2750</v>
       </c>
       <c r="C832" t="n">
-        <v>24752</v>
+        <v>26656</v>
       </c>
     </row>
     <row r="833">
@@ -9598,7 +9598,7 @@
         <v>1853</v>
       </c>
       <c r="C833" t="n">
-        <v>80470</v>
+        <v>86660</v>
       </c>
     </row>
     <row r="834">
@@ -9609,7 +9609,7 @@
         <v>854</v>
       </c>
       <c r="C834" t="n">
-        <v>68094</v>
+        <v>73332</v>
       </c>
     </row>
     <row r="835">
@@ -9620,7 +9620,7 @@
         <v>818</v>
       </c>
       <c r="C835" t="n">
-        <v>244517</v>
+        <v>263326</v>
       </c>
     </row>
     <row r="836">
@@ -9631,7 +9631,7 @@
         <v>2787</v>
       </c>
       <c r="C836" t="n">
-        <v>80476.24000000001</v>
+        <v>86666.71000000001</v>
       </c>
     </row>
     <row r="837">
@@ -9642,7 +9642,7 @@
         <v>2684</v>
       </c>
       <c r="C837" t="n">
-        <v>60047</v>
+        <v>64666</v>
       </c>
     </row>
     <row r="838">
@@ -9653,7 +9653,7 @@
         <v>2653</v>
       </c>
       <c r="C838" t="n">
-        <v>74282</v>
+        <v>79996</v>
       </c>
     </row>
     <row r="839">
@@ -9664,7 +9664,7 @@
         <v>2803</v>
       </c>
       <c r="C839" t="n">
-        <v>73658</v>
+        <v>79324</v>
       </c>
     </row>
     <row r="840">
@@ -9675,7 +9675,7 @@
         <v>2659</v>
       </c>
       <c r="C840" t="n">
-        <v>76154</v>
+        <v>82012</v>
       </c>
     </row>
     <row r="841">
@@ -9686,7 +9686,7 @@
         <v>2753</v>
       </c>
       <c r="C841" t="n">
-        <v>46423</v>
+        <v>49994</v>
       </c>
     </row>
     <row r="842">
@@ -9697,7 +9697,7 @@
         <v>2811</v>
       </c>
       <c r="C842" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="843">
@@ -9708,7 +9708,7 @@
         <v>2762</v>
       </c>
       <c r="C843" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="844">
@@ -9719,7 +9719,7 @@
         <v>2702</v>
       </c>
       <c r="C844" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="845">
@@ -9730,7 +9730,7 @@
         <v>104</v>
       </c>
       <c r="C845" t="n">
-        <v>185705</v>
+        <v>199990</v>
       </c>
     </row>
     <row r="846">
@@ -9741,7 +9741,7 @@
         <v>816</v>
       </c>
       <c r="C846" t="n">
-        <v>165815</v>
+        <v>178570</v>
       </c>
     </row>
     <row r="847">
@@ -9752,7 +9752,7 @@
         <v>1344</v>
       </c>
       <c r="C847" t="n">
-        <v>86658</v>
+        <v>93324</v>
       </c>
     </row>
     <row r="848">
@@ -9763,7 +9763,7 @@
         <v>951</v>
       </c>
       <c r="C848" t="n">
-        <v>71188</v>
+        <v>76664</v>
       </c>
     </row>
     <row r="849">
@@ -9774,7 +9774,7 @@
         <v>2449</v>
       </c>
       <c r="C849" t="n">
-        <v>74282</v>
+        <v>79996</v>
       </c>
     </row>
     <row r="850">
@@ -9785,7 +9785,7 @@
         <v>2709</v>
       </c>
       <c r="C850" t="n">
-        <v>111423</v>
+        <v>119994</v>
       </c>
     </row>
     <row r="851">
@@ -9796,7 +9796,7 @@
         <v>1293</v>
       </c>
       <c r="C851" t="n">
-        <v>247611</v>
+        <v>266658</v>
       </c>
     </row>
     <row r="852">
@@ -9829,7 +9829,7 @@
         <v>619</v>
       </c>
       <c r="C854" t="n">
-        <v>167505</v>
+        <v>180390</v>
       </c>
     </row>
     <row r="855">
@@ -9840,7 +9840,7 @@
         <v>2551</v>
       </c>
       <c r="C855" t="n">
-        <v>12675</v>
+        <v>13650</v>
       </c>
     </row>
     <row r="856">
@@ -9851,7 +9851,7 @@
         <v>2190</v>
       </c>
       <c r="C856" t="n">
-        <v>129376</v>
+        <v>139328</v>
       </c>
     </row>
     <row r="857">
@@ -9862,7 +9862,7 @@
         <v>2793</v>
       </c>
       <c r="C857" t="n">
-        <v>12380.96</v>
+        <v>13333.34</v>
       </c>
     </row>
     <row r="858">
@@ -9873,7 +9873,7 @@
         <v>2687</v>
       </c>
       <c r="C858" t="n">
-        <v>61904.8</v>
+        <v>66666.7</v>
       </c>
     </row>
     <row r="859">
@@ -9884,7 +9884,7 @@
         <v>2655</v>
       </c>
       <c r="C859" t="n">
-        <v>71188</v>
+        <v>76664</v>
       </c>
     </row>
     <row r="860">
@@ -9895,7 +9895,7 @@
         <v>2601</v>
       </c>
       <c r="C860" t="n">
-        <v>170235</v>
+        <v>183330</v>
       </c>
     </row>
     <row r="861">
@@ -9906,7 +9906,7 @@
         <v>2745</v>
       </c>
       <c r="C861" t="n">
-        <v>68094</v>
+        <v>73332</v>
       </c>
     </row>
     <row r="862">
@@ -9917,7 +9917,7 @@
         <v>794</v>
       </c>
       <c r="C862" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="863">
@@ -9928,7 +9928,7 @@
         <v>2586</v>
       </c>
       <c r="C863" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="864">
@@ -9939,7 +9939,7 @@
         <v>766</v>
       </c>
       <c r="C864" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="865">
@@ -9950,7 +9950,7 @@
         <v>966</v>
       </c>
       <c r="C865" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="866">
@@ -9961,7 +9961,7 @@
         <v>749</v>
       </c>
       <c r="C866" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="867">
@@ -9972,7 +9972,7 @@
         <v>890</v>
       </c>
       <c r="C867" t="n">
-        <v>433329</v>
+        <v>466662</v>
       </c>
     </row>
     <row r="868">
@@ -9983,7 +9983,7 @@
         <v>2584</v>
       </c>
       <c r="C868" t="n">
-        <v>38961</v>
+        <v>41958</v>
       </c>
     </row>
     <row r="869">
@@ -9994,7 +9994,7 @@
         <v>2363</v>
       </c>
       <c r="C869" t="n">
-        <v>89752</v>
+        <v>96656</v>
       </c>
     </row>
     <row r="870">
@@ -10005,7 +10005,7 @@
         <v>768</v>
       </c>
       <c r="C870" t="n">
-        <v>77376</v>
+        <v>83328</v>
       </c>
     </row>
     <row r="871">
@@ -10016,7 +10016,7 @@
         <v>2308</v>
       </c>
       <c r="C871" t="n">
-        <v>126893</v>
+        <v>136654</v>
       </c>
     </row>
     <row r="872">
@@ -10027,7 +10027,7 @@
         <v>1501</v>
       </c>
       <c r="C872" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="873">
@@ -10038,7 +10038,7 @@
         <v>675</v>
       </c>
       <c r="C873" t="n">
-        <v>123799</v>
+        <v>133322</v>
       </c>
     </row>
     <row r="874">
@@ -10049,7 +10049,7 @@
         <v>2783</v>
       </c>
       <c r="C874" t="n">
-        <v>43333.36</v>
+        <v>46666.69</v>
       </c>
     </row>
     <row r="875">
@@ -10060,7 +10060,7 @@
         <v>2757</v>
       </c>
       <c r="C875" t="n">
-        <v>43333.36</v>
+        <v>46666.69</v>
       </c>
     </row>
     <row r="876">
@@ -10071,7 +10071,7 @@
         <v>2266</v>
       </c>
       <c r="C876" t="n">
-        <v>49523.84</v>
+        <v>53333.36</v>
       </c>
     </row>
     <row r="877">
@@ -10082,7 +10082,7 @@
         <v>351</v>
       </c>
       <c r="C877" t="n">
-        <v>117000</v>
+        <v>126000</v>
       </c>
     </row>
     <row r="878">
@@ -10093,7 +10093,7 @@
         <v>2383</v>
       </c>
       <c r="C878" t="n">
-        <v>87077.5</v>
+        <v>93775.75999999999</v>
       </c>
     </row>
     <row r="879">
@@ -10104,7 +10104,7 @@
         <v>1585</v>
       </c>
       <c r="C879" t="n">
-        <v>102180</v>
+        <v>110040</v>
       </c>
     </row>
     <row r="880">
@@ -10115,7 +10115,7 @@
         <v>2330</v>
       </c>
       <c r="C880" t="n">
-        <v>166860.97</v>
+        <v>179696.42</v>
       </c>
     </row>
     <row r="881">
@@ -10126,7 +10126,7 @@
         <v>2413</v>
       </c>
       <c r="C881" t="n">
-        <v>74932</v>
+        <v>80696</v>
       </c>
     </row>
     <row r="882">
@@ -10137,7 +10137,7 @@
         <v>1450</v>
       </c>
       <c r="C882" t="n">
-        <v>168727</v>
+        <v>181706</v>
       </c>
     </row>
     <row r="883">
@@ -10148,7 +10148,7 @@
         <v>626</v>
       </c>
       <c r="C883" t="n">
-        <v>1055052.2</v>
+        <v>1136210.05</v>
       </c>
     </row>
     <row r="884">
@@ -10170,7 +10170,7 @@
         <v>89</v>
       </c>
       <c r="C885" t="n">
-        <v>209352</v>
+        <v>225456</v>
       </c>
     </row>
     <row r="886">
@@ -10181,7 +10181,7 @@
         <v>2146</v>
       </c>
       <c r="C886" t="n">
-        <v>124826</v>
+        <v>134428</v>
       </c>
     </row>
     <row r="887">
@@ -10192,7 +10192,7 @@
         <v>2223</v>
       </c>
       <c r="C887" t="n">
-        <v>81679</v>
+        <v>87962</v>
       </c>
     </row>
     <row r="888">
@@ -10203,7 +10203,7 @@
         <v>2633</v>
       </c>
       <c r="C888" t="n">
-        <v>10245.36</v>
+        <v>11033.44</v>
       </c>
     </row>
     <row r="889">
@@ -10214,7 +10214,7 @@
         <v>2577</v>
       </c>
       <c r="C889" t="n">
-        <v>30634.33</v>
+        <v>32990.8</v>
       </c>
     </row>
     <row r="890">
@@ -10236,7 +10236,7 @@
         <v>559</v>
       </c>
       <c r="C891" t="n">
-        <v>154752</v>
+        <v>166656</v>
       </c>
     </row>
     <row r="892">
@@ -10247,7 +10247,7 @@
         <v>42</v>
       </c>
       <c r="C892" t="n">
-        <v>1181141</v>
+        <v>1271998</v>
       </c>
     </row>
     <row r="893">
@@ -10258,7 +10258,7 @@
         <v>663</v>
       </c>
       <c r="C893" t="n">
-        <v>165282</v>
+        <v>177996</v>
       </c>
     </row>
     <row r="894">
@@ -10280,7 +10280,7 @@
         <v>353</v>
       </c>
       <c r="C895" t="n">
-        <v>212921.96</v>
+        <v>229300.56</v>
       </c>
     </row>
     <row r="896">
@@ -10302,7 +10302,7 @@
         <v>2548</v>
       </c>
       <c r="C897" t="n">
-        <v>36218</v>
+        <v>39004</v>
       </c>
     </row>
     <row r="898">
@@ -10313,7 +10313,7 @@
         <v>2552</v>
       </c>
       <c r="C898" t="n">
-        <v>18304</v>
+        <v>19712</v>
       </c>
     </row>
     <row r="899">
@@ -10324,7 +10324,7 @@
         <v>1756</v>
       </c>
       <c r="C899" t="n">
-        <v>270218</v>
+        <v>291004</v>
       </c>
     </row>
     <row r="900">
@@ -10335,7 +10335,7 @@
         <v>2546</v>
       </c>
       <c r="C900" t="n">
-        <v>14768</v>
+        <v>15904</v>
       </c>
     </row>
     <row r="901">
@@ -10346,7 +10346,7 @@
         <v>2561</v>
       </c>
       <c r="C901" t="n">
-        <v>9100</v>
+        <v>9800</v>
       </c>
     </row>
     <row r="902">
@@ -10357,7 +10357,7 @@
         <v>415</v>
       </c>
       <c r="C902" t="n">
-        <v>327860</v>
+        <v>353080</v>
       </c>
     </row>
     <row r="903">
@@ -10368,7 +10368,7 @@
         <v>2727</v>
       </c>
       <c r="C903" t="n">
-        <v>27857.2</v>
+        <v>30000.05</v>
       </c>
     </row>
     <row r="904">
@@ -10379,7 +10379,7 @@
         <v>609</v>
       </c>
       <c r="C904" t="n">
-        <v>136190.48</v>
+        <v>146666.67</v>
       </c>
     </row>
     <row r="905">
@@ -10390,7 +10390,7 @@
         <v>1876</v>
       </c>
       <c r="C905" t="n">
-        <v>43333.36</v>
+        <v>46666.69</v>
       </c>
     </row>
     <row r="906">
@@ -10401,7 +10401,7 @@
         <v>2718</v>
       </c>
       <c r="C906" t="n">
-        <v>43329</v>
+        <v>46662</v>
       </c>
     </row>
     <row r="907">
@@ -10412,7 +10412,7 @@
         <v>2652</v>
       </c>
       <c r="C907" t="n">
-        <v>80470</v>
+        <v>86660</v>
       </c>
     </row>
     <row r="908">
@@ -10423,7 +10423,7 @@
         <v>952</v>
       </c>
       <c r="C908" t="n">
-        <v>55705</v>
+        <v>59990</v>
       </c>
     </row>
     <row r="909">
@@ -10434,7 +10434,7 @@
         <v>1642</v>
       </c>
       <c r="C909" t="n">
-        <v>164047</v>
+        <v>176666</v>
       </c>
     </row>
     <row r="910">
@@ -10445,7 +10445,7 @@
         <v>744</v>
       </c>
       <c r="C910" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="911">
@@ -10456,7 +10456,7 @@
         <v>2323</v>
       </c>
       <c r="C911" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="912">
@@ -10467,7 +10467,7 @@
         <v>970</v>
       </c>
       <c r="C912" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="913">
@@ -10478,7 +10478,7 @@
         <v>2629</v>
       </c>
       <c r="C913" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="914">
@@ -10489,7 +10489,7 @@
         <v>933</v>
       </c>
       <c r="C914" t="n">
-        <v>50440</v>
+        <v>54320</v>
       </c>
     </row>
     <row r="915">
@@ -10500,7 +10500,7 @@
         <v>634</v>
       </c>
       <c r="C915" t="n">
-        <v>340470</v>
+        <v>366660</v>
       </c>
     </row>
     <row r="916">
@@ -10511,7 +10511,7 @@
         <v>2711</v>
       </c>
       <c r="C916" t="n">
-        <v>32190.56</v>
+        <v>34666.74</v>
       </c>
     </row>
     <row r="917">
@@ -10522,7 +10522,7 @@
         <v>1254</v>
       </c>
       <c r="C917" t="n">
-        <v>120404.88</v>
+        <v>129666.77</v>
       </c>
     </row>
     <row r="918">
@@ -10533,7 +10533,7 @@
         <v>2773</v>
       </c>
       <c r="C918" t="n">
-        <v>50142.96</v>
+        <v>54000.09</v>
       </c>
     </row>
     <row r="919">
@@ -10577,7 +10577,7 @@
         <v>530</v>
       </c>
       <c r="C922" t="n">
-        <v>151086</v>
+        <v>162708</v>
       </c>
     </row>
     <row r="923">
@@ -10588,7 +10588,7 @@
         <v>1810</v>
       </c>
       <c r="C923" t="n">
-        <v>22347</v>
+        <v>24066</v>
       </c>
     </row>
     <row r="924">
@@ -10599,7 +10599,7 @@
         <v>2045</v>
       </c>
       <c r="C924" t="n">
-        <v>179255.98</v>
+        <v>193044.89</v>
       </c>
     </row>
     <row r="925">
@@ -10621,7 +10621,7 @@
         <v>2755</v>
       </c>
       <c r="C926" t="n">
-        <v>37142.88</v>
+        <v>40000.02</v>
       </c>
     </row>
     <row r="927">
@@ -10643,7 +10643,7 @@
         <v>2142</v>
       </c>
       <c r="C928" t="n">
-        <v>29770</v>
+        <v>32060</v>
       </c>
     </row>
     <row r="929">
@@ -10665,7 +10665,7 @@
         <v>2641</v>
       </c>
       <c r="C930" t="n">
-        <v>89752</v>
+        <v>96656</v>
       </c>
     </row>
     <row r="931">
@@ -10676,7 +10676,7 @@
         <v>1317</v>
       </c>
       <c r="C931" t="n">
-        <v>185705</v>
+        <v>199990</v>
       </c>
     </row>
     <row r="932">
@@ -10709,7 +10709,7 @@
         <v>2463</v>
       </c>
       <c r="C934" t="n">
-        <v>192036</v>
+        <v>206808</v>
       </c>
     </row>
     <row r="935">
@@ -10720,7 +10720,7 @@
         <v>40</v>
       </c>
       <c r="C935" t="n">
-        <v>145054</v>
+        <v>156212</v>
       </c>
     </row>
     <row r="936">
@@ -10731,7 +10731,7 @@
         <v>1478</v>
       </c>
       <c r="C936" t="n">
-        <v>358930</v>
+        <v>386540</v>
       </c>
     </row>
     <row r="937">
@@ -10742,7 +10742,7 @@
         <v>2026</v>
       </c>
       <c r="C937" t="n">
-        <v>176421.05</v>
+        <v>189991.89</v>
       </c>
     </row>
     <row r="938">
@@ -10764,7 +10764,7 @@
         <v>2554</v>
       </c>
       <c r="C939" t="n">
-        <v>15197</v>
+        <v>16366</v>
       </c>
     </row>
     <row r="940">
@@ -10775,7 +10775,7 @@
         <v>1117</v>
       </c>
       <c r="C940" t="n">
-        <v>215358</v>
+        <v>231924</v>
       </c>
     </row>
     <row r="941">
@@ -10786,7 +10786,7 @@
         <v>2549</v>
       </c>
       <c r="C941" t="n">
-        <v>17550</v>
+        <v>18900</v>
       </c>
     </row>
     <row r="942">
@@ -10797,7 +10797,7 @@
         <v>2791</v>
       </c>
       <c r="C942" t="n">
-        <v>61100</v>
+        <v>65800</v>
       </c>
     </row>
     <row r="943">
@@ -10808,7 +10808,7 @@
         <v>2544</v>
       </c>
       <c r="C943" t="n">
-        <v>37141</v>
+        <v>39998</v>
       </c>
     </row>
     <row r="944">
@@ -10819,7 +10819,7 @@
         <v>1492</v>
       </c>
       <c r="C944" t="n">
-        <v>49517</v>
+        <v>53326</v>
       </c>
     </row>
     <row r="945">
@@ -10830,7 +10830,7 @@
         <v>2131</v>
       </c>
       <c r="C945" t="n">
-        <v>86658</v>
+        <v>93324</v>
       </c>
     </row>
     <row r="946">
@@ -10841,7 +10841,7 @@
         <v>2663</v>
       </c>
       <c r="C946" t="n">
-        <v>170235</v>
+        <v>183330</v>
       </c>
     </row>
     <row r="947">
@@ -10852,7 +10852,7 @@
         <v>793</v>
       </c>
       <c r="C947" t="n">
-        <v>23179</v>
+        <v>24962</v>
       </c>
     </row>
     <row r="948">
@@ -10863,7 +10863,7 @@
         <v>2809</v>
       </c>
       <c r="C948" t="n">
-        <v>42523</v>
+        <v>45794</v>
       </c>
     </row>
     <row r="949">
@@ -10874,7 +10874,7 @@
         <v>931</v>
       </c>
       <c r="C949" t="n">
-        <v>58448</v>
+        <v>62944</v>
       </c>
     </row>
     <row r="950">
@@ -10885,7 +10885,7 @@
         <v>2345</v>
       </c>
       <c r="C950" t="n">
-        <v>38961</v>
+        <v>41958</v>
       </c>
     </row>
     <row r="951">
@@ -10896,7 +10896,7 @@
         <v>1381</v>
       </c>
       <c r="C951" t="n">
-        <v>182611</v>
+        <v>196658</v>
       </c>
     </row>
     <row r="952">
@@ -10907,7 +10907,7 @@
         <v>2124</v>
       </c>
       <c r="C952" t="n">
-        <v>204282</v>
+        <v>219996</v>
       </c>
     </row>
     <row r="953">
@@ -10918,7 +10918,7 @@
         <v>363</v>
       </c>
       <c r="C953" t="n">
-        <v>207376</v>
+        <v>223328</v>
       </c>
     </row>
     <row r="954">
@@ -10929,7 +10929,7 @@
         <v>703</v>
       </c>
       <c r="C954" t="n">
-        <v>142376</v>
+        <v>153328</v>
       </c>
     </row>
     <row r="955">
@@ -10940,7 +10940,7 @@
         <v>2748</v>
       </c>
       <c r="C955" t="n">
-        <v>43333.36</v>
+        <v>46666.69</v>
       </c>
     </row>
     <row r="956">
@@ -10951,7 +10951,7 @@
         <v>2673</v>
       </c>
       <c r="C956" t="n">
-        <v>61893</v>
+        <v>66654</v>
       </c>
     </row>
     <row r="957">
@@ -10962,7 +10962,7 @@
         <v>2118</v>
       </c>
       <c r="C957" t="n">
-        <v>145992.22</v>
+        <v>157222.39</v>
       </c>
     </row>
     <row r="958">
@@ -10973,7 +10973,7 @@
         <v>2325</v>
       </c>
       <c r="C958" t="n">
-        <v>98774</v>
+        <v>106372</v>
       </c>
     </row>
     <row r="959">
@@ -10984,7 +10984,7 @@
         <v>2678</v>
       </c>
       <c r="C959" t="n">
-        <v>210487.91</v>
+        <v>226679.28</v>
       </c>
     </row>
     <row r="960">
@@ -10995,7 +10995,7 @@
         <v>1906</v>
       </c>
       <c r="C960" t="n">
-        <v>70722.32000000001</v>
+        <v>76162.49000000001</v>
       </c>
     </row>
     <row r="961">
@@ -11006,7 +11006,7 @@
         <v>2607</v>
       </c>
       <c r="C961" t="n">
-        <v>28476.24</v>
+        <v>30666.71</v>
       </c>
     </row>
     <row r="962">
@@ -11017,7 +11017,7 @@
         <v>2251</v>
       </c>
       <c r="C962" t="n">
-        <v>132678</v>
+        <v>142884</v>
       </c>
     </row>
     <row r="963">
@@ -11028,7 +11028,7 @@
         <v>1116</v>
       </c>
       <c r="C963" t="n">
-        <v>157014</v>
+        <v>169092</v>
       </c>
     </row>
     <row r="964">
@@ -11039,7 +11039,7 @@
         <v>2651</v>
       </c>
       <c r="C964" t="n">
-        <v>104689</v>
+        <v>112742</v>
       </c>
     </row>
     <row r="965">
@@ -11050,7 +11050,7 @@
         <v>1063</v>
       </c>
       <c r="C965" t="n">
-        <v>225043</v>
+        <v>242354</v>
       </c>
     </row>
     <row r="966">
@@ -11061,7 +11061,7 @@
         <v>2580</v>
       </c>
       <c r="C966" t="n">
-        <v>20769.12</v>
+        <v>22366.73</v>
       </c>
     </row>
     <row r="967">
@@ -11083,7 +11083,7 @@
         <v>2141</v>
       </c>
       <c r="C968" t="n">
-        <v>17641</v>
+        <v>18998</v>
       </c>
     </row>
     <row r="969">
@@ -11105,7 +11105,7 @@
         <v>2660</v>
       </c>
       <c r="C970" t="n">
-        <v>185705</v>
+        <v>199990</v>
       </c>
     </row>
     <row r="971">
@@ -11127,7 +11127,7 @@
         <v>953</v>
       </c>
       <c r="C972" t="n">
-        <v>423839</v>
+        <v>456442</v>
       </c>
     </row>
     <row r="973">
@@ -11138,7 +11138,7 @@
         <v>483</v>
       </c>
       <c r="C973" t="n">
-        <v>274235</v>
+        <v>295330</v>
       </c>
     </row>
     <row r="974">
@@ -11149,7 +11149,7 @@
         <v>525</v>
       </c>
       <c r="C974" t="n">
-        <v>130000</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="975">
@@ -11171,7 +11171,7 @@
         <v>424</v>
       </c>
       <c r="C976" t="n">
-        <v>143572</v>
+        <v>154616</v>
       </c>
     </row>
     <row r="977">
@@ -11193,7 +11193,7 @@
         <v>2550</v>
       </c>
       <c r="C978" t="n">
-        <v>37752</v>
+        <v>40656</v>
       </c>
     </row>
     <row r="979">
@@ -11204,7 +11204,7 @@
         <v>2555</v>
       </c>
       <c r="C979" t="n">
-        <v>25688</v>
+        <v>27664</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 10:10:04
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -6793,7 +6793,7 @@
         <v>2163</v>
       </c>
       <c r="C578" t="n">
-        <v>119988</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="579">
@@ -6804,7 +6804,7 @@
         <v>2621</v>
       </c>
       <c r="C579" t="n">
-        <v>59994</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="580">
@@ -6815,7 +6815,7 @@
         <v>2737</v>
       </c>
       <c r="C580" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="581">
@@ -6826,7 +6826,7 @@
         <v>2090</v>
       </c>
       <c r="C581" t="n">
-        <v>32094</v>
+        <v>37449.33</v>
       </c>
     </row>
     <row r="582">
@@ -6837,7 +6837,7 @@
         <v>2310</v>
       </c>
       <c r="C582" t="n">
-        <v>58878</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="583">
@@ -6848,7 +6848,7 @@
         <v>27</v>
       </c>
       <c r="C583" t="n">
-        <v>85698</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="584">
@@ -6859,7 +6859,7 @@
         <v>522</v>
       </c>
       <c r="C584" t="n">
-        <v>171414</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="585">
@@ -6870,7 +6870,7 @@
         <v>2676</v>
       </c>
       <c r="C585" t="n">
-        <v>53946</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="586">
@@ -6881,7 +6881,7 @@
         <v>1380</v>
       </c>
       <c r="C586" t="n">
-        <v>85698</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="587">
@@ -6892,7 +6892,7 @@
         <v>2069</v>
       </c>
       <c r="C587" t="n">
-        <v>154278</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="588">
@@ -6903,7 +6903,7 @@
         <v>2734</v>
       </c>
       <c r="C588" t="n">
-        <v>47196</v>
+        <v>55081.16</v>
       </c>
     </row>
     <row r="589">
@@ -6914,7 +6914,7 @@
         <v>1137</v>
       </c>
       <c r="C589" t="n">
-        <v>531414</v>
+        <v>620000</v>
       </c>
     </row>
     <row r="590">
@@ -6925,7 +6925,7 @@
         <v>631</v>
       </c>
       <c r="C590" t="n">
-        <v>282852</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="591">
@@ -6936,7 +6936,7 @@
         <v>2081</v>
       </c>
       <c r="C591" t="n">
-        <v>115704</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="592">
@@ -6947,7 +6947,7 @@
         <v>2819</v>
       </c>
       <c r="C592" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="593">
@@ -6958,7 +6958,7 @@
         <v>2742</v>
       </c>
       <c r="C593" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="594">
@@ -6980,7 +6980,7 @@
         <v>1499</v>
       </c>
       <c r="C595" t="n">
-        <v>102852</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="596">
@@ -6991,7 +6991,7 @@
         <v>2442</v>
       </c>
       <c r="C596" t="n">
-        <v>66852</v>
+        <v>78000</v>
       </c>
     </row>
     <row r="597">
@@ -7002,7 +7002,7 @@
         <v>2557</v>
       </c>
       <c r="C597" t="n">
-        <v>22086</v>
+        <v>25785.9</v>
       </c>
     </row>
     <row r="598">
@@ -7013,7 +7013,7 @@
         <v>772</v>
       </c>
       <c r="C598" t="n">
-        <v>301698</v>
+        <v>352000</v>
       </c>
     </row>
     <row r="599">
@@ -7024,7 +7024,7 @@
         <v>2728</v>
       </c>
       <c r="C599" t="n">
-        <v>137142.88</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="600">
@@ -7035,7 +7035,7 @@
         <v>1956</v>
       </c>
       <c r="C600" t="n">
-        <v>216411.6</v>
+        <v>252480.18</v>
       </c>
     </row>
     <row r="601">
@@ -7046,7 +7046,7 @@
         <v>2496</v>
       </c>
       <c r="C601" t="n">
-        <v>119988</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="602">
@@ -7057,7 +7057,7 @@
         <v>2261</v>
       </c>
       <c r="C602" t="n">
-        <v>128556</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="603">
@@ -7068,7 +7068,7 @@
         <v>2794</v>
       </c>
       <c r="C603" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="604">
@@ -7079,7 +7079,7 @@
         <v>2769</v>
       </c>
       <c r="C604" t="n">
-        <v>0.88</v>
+        <v>1</v>
       </c>
     </row>
     <row r="605">
@@ -7090,7 +7090,7 @@
         <v>2804</v>
       </c>
       <c r="C605" t="n">
-        <v>81414</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="606">
@@ -7101,7 +7101,7 @@
         <v>2714</v>
       </c>
       <c r="C606" t="n">
-        <v>291420</v>
+        <v>340000</v>
       </c>
     </row>
     <row r="607">
@@ -7112,7 +7112,7 @@
         <v>2375</v>
       </c>
       <c r="C607" t="n">
-        <v>282852</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="608">
@@ -7123,7 +7123,7 @@
         <v>1539</v>
       </c>
       <c r="C608" t="n">
-        <v>145710</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="609">
@@ -7134,7 +7134,7 @@
         <v>2817</v>
       </c>
       <c r="C609" t="n">
-        <v>51426</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="610">
@@ -7145,7 +7145,7 @@
         <v>2784</v>
       </c>
       <c r="C610" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="611">
@@ -7156,7 +7156,7 @@
         <v>2785</v>
       </c>
       <c r="C611" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="612">
@@ -7167,7 +7167,7 @@
         <v>2761</v>
       </c>
       <c r="C612" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="613">
@@ -7178,7 +7178,7 @@
         <v>2721</v>
       </c>
       <c r="C613" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="614">
@@ -7189,7 +7189,7 @@
         <v>2501</v>
       </c>
       <c r="C614" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="615">
@@ -7200,7 +7200,7 @@
         <v>1007</v>
       </c>
       <c r="C615" t="n">
-        <v>162846</v>
+        <v>190000</v>
       </c>
     </row>
     <row r="616">
@@ -7211,7 +7211,7 @@
         <v>1278</v>
       </c>
       <c r="C616" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="617">
@@ -7233,7 +7233,7 @@
         <v>2689</v>
       </c>
       <c r="C618" t="n">
-        <v>53946</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="619">
@@ -7244,7 +7244,7 @@
         <v>20</v>
       </c>
       <c r="C619" t="n">
-        <v>334278</v>
+        <v>390000</v>
       </c>
     </row>
     <row r="620">
@@ -7255,7 +7255,7 @@
         <v>580</v>
       </c>
       <c r="C620" t="n">
-        <v>115704</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="621">
@@ -7266,7 +7266,7 @@
         <v>2802</v>
       </c>
       <c r="C621" t="n">
-        <v>60696</v>
+        <v>70818.64</v>
       </c>
     </row>
     <row r="622">
@@ -7277,7 +7277,7 @@
         <v>1340</v>
       </c>
       <c r="C622" t="n">
-        <v>111420</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="623">
@@ -7288,7 +7288,7 @@
         <v>358</v>
       </c>
       <c r="C623" t="n">
-        <v>304272</v>
+        <v>355000</v>
       </c>
     </row>
     <row r="624">
@@ -7299,7 +7299,7 @@
         <v>636</v>
       </c>
       <c r="C624" t="n">
-        <v>214272</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="625">
@@ -7310,7 +7310,7 @@
         <v>1374</v>
       </c>
       <c r="C625" t="n">
-        <v>145710</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="626">
@@ -7321,7 +7321,7 @@
         <v>2440</v>
       </c>
       <c r="C626" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="627">
@@ -7332,7 +7332,7 @@
         <v>429</v>
       </c>
       <c r="C627" t="n">
-        <v>334278</v>
+        <v>390000</v>
       </c>
     </row>
     <row r="628">
@@ -7343,7 +7343,7 @@
         <v>2015</v>
       </c>
       <c r="C628" t="n">
-        <v>304272</v>
+        <v>355000</v>
       </c>
     </row>
     <row r="629">
@@ -7354,7 +7354,7 @@
         <v>1259</v>
       </c>
       <c r="C629" t="n">
-        <v>85714.3</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="630">
@@ -7365,7 +7365,7 @@
         <v>2346</v>
       </c>
       <c r="C630" t="n">
-        <v>94285.73</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="631">
@@ -7376,7 +7376,7 @@
         <v>2431</v>
       </c>
       <c r="C631" t="n">
-        <v>161136</v>
+        <v>188000</v>
       </c>
     </row>
     <row r="632">
@@ -7387,7 +7387,7 @@
         <v>2792</v>
       </c>
       <c r="C632" t="n">
-        <v>100928.81</v>
+        <v>117757.97</v>
       </c>
     </row>
     <row r="633">
@@ -7398,7 +7398,7 @@
         <v>2114</v>
       </c>
       <c r="C633" t="n">
-        <v>158888.91</v>
+        <v>185371.92</v>
       </c>
     </row>
     <row r="634">
@@ -7409,7 +7409,7 @@
         <v>2359</v>
       </c>
       <c r="C634" t="n">
-        <v>96390.31</v>
+        <v>112466.45</v>
       </c>
     </row>
     <row r="635">
@@ -7420,7 +7420,7 @@
         <v>1142</v>
       </c>
       <c r="C635" t="n">
-        <v>367758</v>
+        <v>429052.25</v>
       </c>
     </row>
     <row r="636">
@@ -7431,7 +7431,7 @@
         <v>569</v>
       </c>
       <c r="C636" t="n">
-        <v>2454786</v>
+        <v>2863931.44</v>
       </c>
     </row>
     <row r="637">
@@ -7464,7 +7464,7 @@
         <v>2333</v>
       </c>
       <c r="C639" t="n">
-        <v>132300</v>
+        <v>154354.21</v>
       </c>
     </row>
     <row r="640">
@@ -7475,7 +7475,7 @@
         <v>2707</v>
       </c>
       <c r="C640" t="n">
-        <v>27471.46</v>
+        <v>32050</v>
       </c>
     </row>
     <row r="641">
@@ -7486,7 +7486,7 @@
         <v>2472</v>
       </c>
       <c r="C641" t="n">
-        <v>45385.74</v>
+        <v>52950</v>
       </c>
     </row>
     <row r="642">
@@ -7530,7 +7530,7 @@
         <v>2498</v>
       </c>
       <c r="C645" t="n">
-        <v>42876</v>
+        <v>50030.36</v>
       </c>
     </row>
     <row r="646">
@@ -7541,7 +7541,7 @@
         <v>2381</v>
       </c>
       <c r="C646" t="n">
-        <v>61254</v>
+        <v>71467.39</v>
       </c>
     </row>
     <row r="647">
@@ -7552,7 +7552,7 @@
         <v>2273</v>
       </c>
       <c r="C647" t="n">
-        <v>163746</v>
+        <v>191055.04</v>
       </c>
     </row>
     <row r="648">
@@ -7563,7 +7563,7 @@
         <v>2647</v>
       </c>
       <c r="C648" t="n">
-        <v>121626</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="649">
@@ -7574,7 +7574,7 @@
         <v>2492</v>
       </c>
       <c r="C649" t="n">
-        <v>121626</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="650">
@@ -7585,7 +7585,7 @@
         <v>2631</v>
       </c>
       <c r="C650" t="n">
-        <v>21042.88</v>
+        <v>24550</v>
       </c>
     </row>
     <row r="651">
@@ -7596,7 +7596,7 @@
         <v>2682</v>
       </c>
       <c r="C651" t="n">
-        <v>128571.45</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="652">
@@ -7607,7 +7607,7 @@
         <v>1075</v>
       </c>
       <c r="C652" t="n">
-        <v>388278</v>
+        <v>453000</v>
       </c>
     </row>
     <row r="653">
@@ -7618,7 +7618,7 @@
         <v>2810</v>
       </c>
       <c r="C653" t="n">
-        <v>119988</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="654">
@@ -7629,7 +7629,7 @@
         <v>2547</v>
       </c>
       <c r="C654" t="n">
-        <v>35262</v>
+        <v>41139.75</v>
       </c>
     </row>
     <row r="655">
@@ -7640,7 +7640,7 @@
         <v>2627</v>
       </c>
       <c r="C655" t="n">
-        <v>20898</v>
+        <v>24394.96</v>
       </c>
     </row>
     <row r="656">
@@ -7662,7 +7662,7 @@
         <v>2562</v>
       </c>
       <c r="C657" t="n">
-        <v>13572</v>
+        <v>15835.33</v>
       </c>
     </row>
     <row r="658">
@@ -7673,7 +7673,7 @@
         <v>1658</v>
       </c>
       <c r="C658" t="n">
-        <v>116568</v>
+        <v>136000</v>
       </c>
     </row>
     <row r="659">
@@ -7684,7 +7684,7 @@
         <v>1996</v>
       </c>
       <c r="C659" t="n">
-        <v>300636</v>
+        <v>350745</v>
       </c>
     </row>
     <row r="660">
@@ -7695,7 +7695,7 @@
         <v>2674</v>
       </c>
       <c r="C660" t="n">
-        <v>222840</v>
+        <v>260000</v>
       </c>
     </row>
     <row r="661">
@@ -7706,7 +7706,7 @@
         <v>2667</v>
       </c>
       <c r="C661" t="n">
-        <v>39171.46</v>
+        <v>45700</v>
       </c>
     </row>
     <row r="662">
@@ -7728,7 +7728,7 @@
         <v>1834</v>
       </c>
       <c r="C663" t="n">
-        <v>100278</v>
+        <v>117010.45</v>
       </c>
     </row>
     <row r="664">
@@ -7739,7 +7739,7 @@
         <v>2109</v>
       </c>
       <c r="C664" t="n">
-        <v>80142.86</v>
+        <v>93500</v>
       </c>
     </row>
     <row r="665">
@@ -7783,7 +7783,7 @@
         <v>630</v>
       </c>
       <c r="C668" t="n">
-        <v>23148</v>
+        <v>27020.83</v>
       </c>
     </row>
     <row r="669">
@@ -7794,7 +7794,7 @@
         <v>2197</v>
       </c>
       <c r="C669" t="n">
-        <v>171414</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="670">
@@ -7816,7 +7816,7 @@
         <v>1983</v>
       </c>
       <c r="C671" t="n">
-        <v>496980</v>
+        <v>579828.27</v>
       </c>
     </row>
     <row r="672">
@@ -7827,7 +7827,7 @@
         <v>941</v>
       </c>
       <c r="C672" t="n">
-        <v>303238.25</v>
+        <v>353777.93</v>
       </c>
     </row>
     <row r="673">
@@ -7849,7 +7849,7 @@
         <v>2556</v>
       </c>
       <c r="C674" t="n">
-        <v>30942</v>
+        <v>36110.97</v>
       </c>
     </row>
     <row r="675">
@@ -7871,7 +7871,7 @@
         <v>1993</v>
       </c>
       <c r="C676" t="n">
-        <v>298188</v>
+        <v>347896.96</v>
       </c>
     </row>
     <row r="677">
@@ -7882,7 +7882,7 @@
         <v>949</v>
       </c>
       <c r="C677" t="n">
-        <v>84132</v>
+        <v>98163.42</v>
       </c>
     </row>
     <row r="678">
@@ -7893,7 +7893,7 @@
         <v>1298</v>
       </c>
       <c r="C678" t="n">
-        <v>962784</v>
+        <v>1123255</v>
       </c>
     </row>
     <row r="679">
@@ -7904,7 +7904,7 @@
         <v>2729</v>
       </c>
       <c r="C679" t="n">
-        <v>42840</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="680">
@@ -7915,7 +7915,7 @@
         <v>1873</v>
       </c>
       <c r="C680" t="n">
-        <v>273420</v>
+        <v>319000</v>
       </c>
     </row>
     <row r="681">
@@ -7926,7 +7926,7 @@
         <v>1466</v>
       </c>
       <c r="C681" t="n">
-        <v>338562</v>
+        <v>395000</v>
       </c>
     </row>
     <row r="682">
@@ -7937,7 +7937,7 @@
         <v>2671</v>
       </c>
       <c r="C682" t="n">
-        <v>68562</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="683">
@@ -7948,7 +7948,7 @@
         <v>2786</v>
       </c>
       <c r="C683" t="n">
-        <v>59994</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="684">
@@ -7959,7 +7959,7 @@
         <v>2073</v>
       </c>
       <c r="C684" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="685">
@@ -7970,7 +7970,7 @@
         <v>2583</v>
       </c>
       <c r="C685" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="686">
@@ -7981,7 +7981,7 @@
         <v>2796</v>
       </c>
       <c r="C686" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="687">
@@ -7992,7 +7992,7 @@
         <v>1384</v>
       </c>
       <c r="C687" t="n">
-        <v>385704</v>
+        <v>450000</v>
       </c>
     </row>
     <row r="688">
@@ -8003,7 +8003,7 @@
         <v>132</v>
       </c>
       <c r="C688" t="n">
-        <v>642852</v>
+        <v>750000</v>
       </c>
     </row>
     <row r="689">
@@ -8014,7 +8014,7 @@
         <v>1518</v>
       </c>
       <c r="C689" t="n">
-        <v>299988</v>
+        <v>350000</v>
       </c>
     </row>
     <row r="690">
@@ -8025,7 +8025,7 @@
         <v>438</v>
       </c>
       <c r="C690" t="n">
-        <v>132840</v>
+        <v>155000</v>
       </c>
     </row>
     <row r="691">
@@ -8036,7 +8036,7 @@
         <v>2716</v>
       </c>
       <c r="C691" t="n">
-        <v>74178</v>
+        <v>86556.11</v>
       </c>
     </row>
     <row r="692">
@@ -8047,7 +8047,7 @@
         <v>14</v>
       </c>
       <c r="C692" t="n">
-        <v>372852</v>
+        <v>435000</v>
       </c>
     </row>
     <row r="693">
@@ -8058,7 +8058,7 @@
         <v>535</v>
       </c>
       <c r="C693" t="n">
-        <v>325710</v>
+        <v>380000</v>
       </c>
     </row>
     <row r="694">
@@ -8069,7 +8069,7 @@
         <v>2795</v>
       </c>
       <c r="C694" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="695">
@@ -8080,7 +8080,7 @@
         <v>1456</v>
       </c>
       <c r="C695" t="n">
-        <v>660240</v>
+        <v>770288.58</v>
       </c>
     </row>
     <row r="696">
@@ -8091,7 +8091,7 @@
         <v>2249</v>
       </c>
       <c r="C696" t="n">
-        <v>167418</v>
+        <v>195323.18</v>
       </c>
     </row>
     <row r="697">
@@ -8102,7 +8102,7 @@
         <v>2394</v>
       </c>
       <c r="C697" t="n">
-        <v>132048</v>
+        <v>154057.72</v>
       </c>
     </row>
     <row r="698">
@@ -8113,7 +8113,7 @@
         <v>2507</v>
       </c>
       <c r="C698" t="n">
-        <v>78694.58</v>
+        <v>91811.37</v>
       </c>
     </row>
     <row r="699">
@@ -8124,7 +8124,7 @@
         <v>2697</v>
       </c>
       <c r="C699" t="n">
-        <v>165044.1</v>
+        <v>192554.28</v>
       </c>
     </row>
     <row r="700">
@@ -8135,7 +8135,7 @@
         <v>2698</v>
       </c>
       <c r="C700" t="n">
-        <v>104719.83</v>
+        <v>122177.3</v>
       </c>
     </row>
     <row r="701">
@@ -8146,7 +8146,7 @@
         <v>2510</v>
       </c>
       <c r="C701" t="n">
-        <v>475920</v>
+        <v>555244.09</v>
       </c>
     </row>
     <row r="702">
@@ -8157,7 +8157,7 @@
         <v>2613</v>
       </c>
       <c r="C702" t="n">
-        <v>153576</v>
+        <v>179192.41</v>
       </c>
     </row>
     <row r="703">
@@ -8168,7 +8168,7 @@
         <v>2820</v>
       </c>
       <c r="C703" t="n">
-        <v>154285.74</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="704">
@@ -8190,7 +8190,7 @@
         <v>1871</v>
       </c>
       <c r="C705" t="n">
-        <v>151506</v>
+        <v>176760.47</v>
       </c>
     </row>
     <row r="706">
@@ -8223,7 +8223,7 @@
         <v>2145</v>
       </c>
       <c r="C708" t="n">
-        <v>110952</v>
+        <v>129458.37</v>
       </c>
     </row>
     <row r="709">
@@ -8234,7 +8234,7 @@
         <v>2574</v>
       </c>
       <c r="C709" t="n">
-        <v>110952</v>
+        <v>129458.37</v>
       </c>
     </row>
     <row r="710">
@@ -8245,7 +8245,7 @@
         <v>2411</v>
       </c>
       <c r="C710" t="n">
-        <v>121626</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="711">
@@ -8256,7 +8256,7 @@
         <v>2692</v>
       </c>
       <c r="C711" t="n">
-        <v>64285.74</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="712">
@@ -8267,7 +8267,7 @@
         <v>945</v>
       </c>
       <c r="C712" t="n">
-        <v>242858.18</v>
+        <v>283334.51</v>
       </c>
     </row>
     <row r="713">
@@ -8289,7 +8289,7 @@
         <v>664</v>
       </c>
       <c r="C714" t="n">
-        <v>229698</v>
+        <v>268000</v>
       </c>
     </row>
     <row r="715">
@@ -8311,7 +8311,7 @@
         <v>947</v>
       </c>
       <c r="C716" t="n">
-        <v>372463.42</v>
+        <v>434540.65</v>
       </c>
     </row>
     <row r="717">
@@ -8333,7 +8333,7 @@
         <v>2279</v>
       </c>
       <c r="C718" t="n">
-        <v>198792</v>
+        <v>231931.31</v>
       </c>
     </row>
     <row r="719">
@@ -8344,7 +8344,7 @@
         <v>58</v>
       </c>
       <c r="C719" t="n">
-        <v>198792</v>
+        <v>231931.31</v>
       </c>
     </row>
     <row r="720">
@@ -8355,7 +8355,7 @@
         <v>2648</v>
       </c>
       <c r="C720" t="n">
-        <v>124272</v>
+        <v>145000</v>
       </c>
     </row>
     <row r="721">
@@ -8377,7 +8377,7 @@
         <v>2558</v>
       </c>
       <c r="C722" t="n">
-        <v>25758</v>
+        <v>30065.72</v>
       </c>
     </row>
     <row r="723">
@@ -8388,7 +8388,7 @@
         <v>2245</v>
       </c>
       <c r="C723" t="n">
-        <v>198792</v>
+        <v>231931.31</v>
       </c>
     </row>
     <row r="724">
@@ -8399,7 +8399,7 @@
         <v>1064</v>
       </c>
       <c r="C724" t="n">
-        <v>513738</v>
+        <v>599374.29</v>
       </c>
     </row>
     <row r="725">
@@ -8410,7 +8410,7 @@
         <v>1293</v>
       </c>
       <c r="C725" t="n">
-        <v>342846</v>
+        <v>400000</v>
       </c>
     </row>
     <row r="726">
@@ -8421,7 +8421,7 @@
         <v>360</v>
       </c>
       <c r="C726" t="n">
-        <v>428562</v>
+        <v>500000</v>
       </c>
     </row>
     <row r="727">
@@ -8432,7 +8432,7 @@
         <v>2767</v>
       </c>
       <c r="C727" t="n">
-        <v>165366</v>
+        <v>192936.84</v>
       </c>
     </row>
     <row r="728">
@@ -8443,7 +8443,7 @@
         <v>781</v>
       </c>
       <c r="C728" t="n">
-        <v>111420</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="729">
@@ -8454,7 +8454,7 @@
         <v>1020</v>
       </c>
       <c r="C729" t="n">
-        <v>72846</v>
+        <v>85000</v>
       </c>
     </row>
     <row r="730">
@@ -8476,7 +8476,7 @@
         <v>2258</v>
       </c>
       <c r="C731" t="n">
-        <v>68571.44</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="732">
@@ -8487,7 +8487,7 @@
         <v>2744</v>
       </c>
       <c r="C732" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="733">
@@ -8498,7 +8498,7 @@
         <v>2758</v>
       </c>
       <c r="C733" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="734">
@@ -8509,7 +8509,7 @@
         <v>2772</v>
       </c>
       <c r="C734" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="735">
@@ -8520,7 +8520,7 @@
         <v>2797</v>
       </c>
       <c r="C735" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="736">
@@ -8531,7 +8531,7 @@
         <v>2815</v>
       </c>
       <c r="C736" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="737">
@@ -8542,7 +8542,7 @@
         <v>1869</v>
       </c>
       <c r="C737" t="n">
-        <v>195426</v>
+        <v>228000</v>
       </c>
     </row>
     <row r="738">
@@ -8553,7 +8553,7 @@
         <v>452</v>
       </c>
       <c r="C738" t="n">
-        <v>222840</v>
+        <v>260000</v>
       </c>
     </row>
     <row r="739">
@@ -8564,7 +8564,7 @@
         <v>2178</v>
       </c>
       <c r="C739" t="n">
-        <v>252846</v>
+        <v>295000</v>
       </c>
     </row>
     <row r="740">
@@ -8575,7 +8575,7 @@
         <v>1308</v>
       </c>
       <c r="C740" t="n">
-        <v>136532.22</v>
+        <v>159305.68</v>
       </c>
     </row>
     <row r="741">
@@ -8586,7 +8586,7 @@
         <v>2107</v>
       </c>
       <c r="C741" t="n">
-        <v>239013.79</v>
+        <v>278855.26</v>
       </c>
     </row>
     <row r="742">
@@ -8597,7 +8597,7 @@
         <v>2211</v>
       </c>
       <c r="C742" t="n">
-        <v>191836.81</v>
+        <v>223814.43</v>
       </c>
     </row>
     <row r="743">
@@ -8608,7 +8608,7 @@
         <v>2567</v>
       </c>
       <c r="C743" t="n">
-        <v>141480</v>
+        <v>165061.84</v>
       </c>
     </row>
     <row r="744">
@@ -8619,7 +8619,7 @@
         <v>2680</v>
       </c>
       <c r="C744" t="n">
-        <v>92640.16</v>
+        <v>108086.81</v>
       </c>
     </row>
     <row r="745">
@@ -8630,7 +8630,7 @@
         <v>2568</v>
       </c>
       <c r="C745" t="n">
-        <v>175212</v>
+        <v>204430.78</v>
       </c>
     </row>
     <row r="746">
@@ -8641,7 +8641,7 @@
         <v>2790</v>
       </c>
       <c r="C746" t="n">
-        <v>54600.04</v>
+        <v>63700</v>
       </c>
     </row>
     <row r="747">
@@ -8663,7 +8663,7 @@
         <v>2250</v>
       </c>
       <c r="C748" t="n">
-        <v>283626</v>
+        <v>330913.83</v>
       </c>
     </row>
     <row r="749">
@@ -8674,7 +8674,7 @@
         <v>2705</v>
       </c>
       <c r="C749" t="n">
-        <v>153576</v>
+        <v>179192.41</v>
       </c>
     </row>
     <row r="750">
@@ -8685,7 +8685,7 @@
         <v>2082</v>
       </c>
       <c r="C750" t="n">
-        <v>142776</v>
+        <v>166573.23</v>
       </c>
     </row>
     <row r="751">
@@ -8696,7 +8696,7 @@
         <v>2183</v>
       </c>
       <c r="C751" t="n">
-        <v>313686</v>
+        <v>365968.86</v>
       </c>
     </row>
     <row r="752">
@@ -8707,7 +8707,7 @@
         <v>2276</v>
       </c>
       <c r="C752" t="n">
-        <v>192042</v>
+        <v>224062.57</v>
       </c>
     </row>
     <row r="753">
@@ -8718,7 +8718,7 @@
         <v>477</v>
       </c>
       <c r="C753" t="n">
-        <v>221706</v>
+        <v>258659.79</v>
       </c>
     </row>
     <row r="754">
@@ -8729,7 +8729,7 @@
         <v>2691</v>
       </c>
       <c r="C754" t="n">
-        <v>115714.29</v>
+        <v>135000</v>
       </c>
     </row>
     <row r="755">
@@ -8740,7 +8740,7 @@
         <v>1289</v>
       </c>
       <c r="C755" t="n">
-        <v>214272</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="756">
@@ -8751,7 +8751,7 @@
         <v>1632</v>
       </c>
       <c r="C756" t="n">
-        <v>214272</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="757">
@@ -8762,7 +8762,7 @@
         <v>2801</v>
       </c>
       <c r="C757" t="n">
-        <v>119988</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="758">
@@ -8773,7 +8773,7 @@
         <v>451</v>
       </c>
       <c r="C758" t="n">
-        <v>214272</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="759">
@@ -8784,7 +8784,7 @@
         <v>1102</v>
       </c>
       <c r="C759" t="n">
-        <v>198792</v>
+        <v>231931.31</v>
       </c>
     </row>
     <row r="760">
@@ -8795,7 +8795,7 @@
         <v>1465</v>
       </c>
       <c r="C760" t="n">
-        <v>308376</v>
+        <v>359789.28</v>
       </c>
     </row>
     <row r="761">
@@ -8806,7 +8806,7 @@
         <v>2649</v>
       </c>
       <c r="C761" t="n">
-        <v>25308</v>
+        <v>29530.75</v>
       </c>
     </row>
     <row r="762">
@@ -8817,7 +8817,7 @@
         <v>400</v>
       </c>
       <c r="C762" t="n">
-        <v>158562</v>
+        <v>185000</v>
       </c>
     </row>
     <row r="763">
@@ -8828,7 +8828,7 @@
         <v>2133</v>
       </c>
       <c r="C763" t="n">
-        <v>689130</v>
+        <v>804000</v>
       </c>
     </row>
     <row r="764">
@@ -8839,7 +8839,7 @@
         <v>767</v>
       </c>
       <c r="C764" t="n">
-        <v>154285.74</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="765">
@@ -8861,7 +8861,7 @@
         <v>2722</v>
       </c>
       <c r="C766" t="n">
-        <v>34272</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="767">
@@ -8872,7 +8872,7 @@
         <v>2566</v>
       </c>
       <c r="C767" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="768">
@@ -8883,7 +8883,7 @@
         <v>2635</v>
       </c>
       <c r="C768" t="n">
-        <v>111420</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="769">
@@ -8894,7 +8894,7 @@
         <v>2726</v>
       </c>
       <c r="C769" t="n">
-        <v>128571.45</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="770">
@@ -8905,7 +8905,7 @@
         <v>2730</v>
       </c>
       <c r="C770" t="n">
-        <v>77142.87</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="771">
@@ -8916,7 +8916,7 @@
         <v>2765</v>
       </c>
       <c r="C771" t="n">
-        <v>81414</v>
+        <v>95000</v>
       </c>
     </row>
     <row r="772">
@@ -8927,7 +8927,7 @@
         <v>2735</v>
       </c>
       <c r="C772" t="n">
-        <v>102852</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="773">
@@ -8938,7 +8938,7 @@
         <v>2816</v>
       </c>
       <c r="C773" t="n">
-        <v>42840</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="774">
@@ -8949,7 +8949,7 @@
         <v>1881</v>
       </c>
       <c r="C774" t="n">
-        <v>58878</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="775">
@@ -8960,7 +8960,7 @@
         <v>595</v>
       </c>
       <c r="C775" t="n">
-        <v>471420</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="776">
@@ -8971,7 +8971,7 @@
         <v>925</v>
       </c>
       <c r="C776" t="n">
-        <v>67446</v>
+        <v>78687.37</v>
       </c>
     </row>
     <row r="777">
@@ -8982,7 +8982,7 @@
         <v>2582</v>
       </c>
       <c r="C777" t="n">
-        <v>74178</v>
+        <v>86556.11</v>
       </c>
     </row>
     <row r="778">
@@ -8993,7 +8993,7 @@
         <v>2637</v>
       </c>
       <c r="C778" t="n">
-        <v>53946</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="779">
@@ -9004,7 +9004,7 @@
         <v>2448</v>
       </c>
       <c r="C779" t="n">
-        <v>59994</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="780">
@@ -9015,7 +9015,7 @@
         <v>2452</v>
       </c>
       <c r="C780" t="n">
-        <v>55710</v>
+        <v>65000</v>
       </c>
     </row>
     <row r="781">
@@ -9026,7 +9026,7 @@
         <v>2362</v>
       </c>
       <c r="C781" t="n">
-        <v>59994</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="782">
@@ -9037,7 +9037,7 @@
         <v>1277</v>
       </c>
       <c r="C782" t="n">
-        <v>188568</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="783">
@@ -9048,7 +9048,7 @@
         <v>1327</v>
       </c>
       <c r="C783" t="n">
-        <v>42840</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="784">
@@ -9059,7 +9059,7 @@
         <v>2599</v>
       </c>
       <c r="C784" t="n">
-        <v>162000</v>
+        <v>189000</v>
       </c>
     </row>
     <row r="785">
@@ -9070,7 +9070,7 @@
         <v>2402</v>
       </c>
       <c r="C785" t="n">
-        <v>558846</v>
+        <v>651994.26</v>
       </c>
     </row>
     <row r="786">
@@ -9081,7 +9081,7 @@
         <v>2085</v>
       </c>
       <c r="C786" t="n">
-        <v>113184</v>
+        <v>132049.47</v>
       </c>
     </row>
     <row r="787">
@@ -9103,7 +9103,7 @@
         <v>2341</v>
       </c>
       <c r="C788" t="n">
-        <v>121626</v>
+        <v>141906.29</v>
       </c>
     </row>
     <row r="789">
@@ -9114,7 +9114,7 @@
         <v>634</v>
       </c>
       <c r="C789" t="n">
-        <v>471420</v>
+        <v>550000</v>
       </c>
     </row>
     <row r="790">
@@ -9125,7 +9125,7 @@
         <v>1372</v>
       </c>
       <c r="C790" t="n">
-        <v>248562</v>
+        <v>290000</v>
       </c>
     </row>
     <row r="791">
@@ -9136,7 +9136,7 @@
         <v>1653</v>
       </c>
       <c r="C791" t="n">
-        <v>287136</v>
+        <v>335000</v>
       </c>
     </row>
     <row r="792">
@@ -9147,7 +9147,7 @@
         <v>1324</v>
       </c>
       <c r="C792" t="n">
-        <v>239994</v>
+        <v>280000</v>
       </c>
     </row>
     <row r="793">
@@ -9158,7 +9158,7 @@
         <v>802</v>
       </c>
       <c r="C793" t="n">
-        <v>64278</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="794">
@@ -9169,7 +9169,7 @@
         <v>2747</v>
       </c>
       <c r="C794" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="795">
@@ -9180,7 +9180,7 @@
         <v>2798</v>
       </c>
       <c r="C795" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="796">
@@ -9191,7 +9191,7 @@
         <v>33</v>
       </c>
       <c r="C796" t="n">
-        <v>333414</v>
+        <v>389000</v>
       </c>
     </row>
     <row r="797">
@@ -9202,7 +9202,7 @@
         <v>783</v>
       </c>
       <c r="C797" t="n">
-        <v>38556</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="798">
@@ -9213,7 +9213,7 @@
         <v>2768</v>
       </c>
       <c r="C798" t="n">
-        <v>286179.06</v>
+        <v>333891.62</v>
       </c>
     </row>
     <row r="799">
@@ -9224,7 +9224,7 @@
         <v>2491</v>
       </c>
       <c r="C799" t="n">
-        <v>93795.94</v>
+        <v>109432.26</v>
       </c>
     </row>
     <row r="800">
@@ -9235,7 +9235,7 @@
         <v>2606</v>
       </c>
       <c r="C800" t="n">
-        <v>202788</v>
+        <v>236588.64</v>
       </c>
     </row>
     <row r="801">
@@ -9246,7 +9246,7 @@
         <v>2799</v>
       </c>
       <c r="C801" t="n">
-        <v>101136.3</v>
+        <v>117999.97</v>
       </c>
     </row>
     <row r="802">
@@ -9257,7 +9257,7 @@
         <v>2571</v>
       </c>
       <c r="C802" t="n">
-        <v>133994.22</v>
+        <v>156347.24</v>
       </c>
     </row>
     <row r="803">
@@ -9268,7 +9268,7 @@
         <v>2696</v>
       </c>
       <c r="C803" t="n">
-        <v>209987.4</v>
+        <v>244994.07</v>
       </c>
     </row>
     <row r="804">
@@ -9279,7 +9279,7 @@
         <v>1907</v>
       </c>
       <c r="C804" t="n">
-        <v>317988</v>
+        <v>371004</v>
       </c>
     </row>
     <row r="805">
@@ -9290,7 +9290,7 @@
         <v>2392</v>
       </c>
       <c r="C805" t="n">
-        <v>142776</v>
+        <v>166573.23</v>
       </c>
     </row>
     <row r="806">
@@ -9301,7 +9301,7 @@
         <v>2706</v>
       </c>
       <c r="C806" t="n">
-        <v>18900.03</v>
+        <v>22050</v>
       </c>
     </row>
     <row r="807">
@@ -9312,7 +9312,7 @@
         <v>2657</v>
       </c>
       <c r="C807" t="n">
-        <v>67885.74000000001</v>
+        <v>79200</v>
       </c>
     </row>
     <row r="808">
@@ -9334,7 +9334,7 @@
         <v>2695</v>
       </c>
       <c r="C809" t="n">
-        <v>36846</v>
+        <v>43005.4</v>
       </c>
     </row>
     <row r="810">
@@ -9345,7 +9345,7 @@
         <v>2700</v>
       </c>
       <c r="C810" t="n">
-        <v>46548</v>
+        <v>54309.5</v>
       </c>
     </row>
     <row r="811">
@@ -9356,7 +9356,7 @@
         <v>1800</v>
       </c>
       <c r="C811" t="n">
-        <v>21600</v>
+        <v>25210.38</v>
       </c>
     </row>
     <row r="812">
@@ -9367,7 +9367,7 @@
         <v>2541</v>
       </c>
       <c r="C812" t="n">
-        <v>181368</v>
+        <v>211614.65</v>
       </c>
     </row>
     <row r="813">
@@ -9378,7 +9378,7 @@
         <v>2365</v>
       </c>
       <c r="C813" t="n">
-        <v>68274</v>
+        <v>79666.69</v>
       </c>
     </row>
     <row r="814">
@@ -9389,7 +9389,7 @@
         <v>1890</v>
       </c>
       <c r="C814" t="n">
-        <v>281249.2</v>
+        <v>328124.02</v>
       </c>
     </row>
     <row r="815">
@@ -9411,7 +9411,7 @@
         <v>1299</v>
       </c>
       <c r="C816" t="n">
-        <v>446004</v>
+        <v>520358.7</v>
       </c>
     </row>
     <row r="817">
@@ -9444,7 +9444,7 @@
         <v>1937</v>
       </c>
       <c r="C819" t="n">
-        <v>222480</v>
+        <v>259575.91</v>
       </c>
     </row>
     <row r="820">
@@ -9455,7 +9455,7 @@
         <v>610</v>
       </c>
       <c r="C820" t="n">
-        <v>703134</v>
+        <v>820332.23</v>
       </c>
     </row>
     <row r="821">
@@ -9466,7 +9466,7 @@
         <v>131</v>
       </c>
       <c r="C821" t="n">
-        <v>350568</v>
+        <v>409000</v>
       </c>
     </row>
     <row r="822">
@@ -9477,7 +9477,7 @@
         <v>2789</v>
       </c>
       <c r="C822" t="n">
-        <v>145710</v>
+        <v>170000</v>
       </c>
     </row>
     <row r="823">
@@ -9510,7 +9510,7 @@
         <v>629</v>
       </c>
       <c r="C825" t="n">
-        <v>376272</v>
+        <v>439000</v>
       </c>
     </row>
     <row r="826">
@@ -9543,7 +9543,7 @@
         <v>285</v>
       </c>
       <c r="C828" t="n">
-        <v>496980</v>
+        <v>579828.27</v>
       </c>
     </row>
     <row r="829">
@@ -9554,7 +9554,7 @@
         <v>2643</v>
       </c>
       <c r="C829" t="n">
-        <v>25308</v>
+        <v>29530.75</v>
       </c>
     </row>
     <row r="830">
@@ -9565,7 +9565,7 @@
         <v>2421</v>
       </c>
       <c r="C830" t="n">
-        <v>48852</v>
+        <v>57000</v>
       </c>
     </row>
     <row r="831">
@@ -9576,7 +9576,7 @@
         <v>571</v>
       </c>
       <c r="C831" t="n">
-        <v>464868</v>
+        <v>542365</v>
       </c>
     </row>
     <row r="832">
@@ -9587,7 +9587,7 @@
         <v>2686</v>
       </c>
       <c r="C832" t="n">
-        <v>111428.59</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="833">
@@ -9598,7 +9598,7 @@
         <v>2494</v>
       </c>
       <c r="C833" t="n">
-        <v>111420</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="834">
@@ -9609,7 +9609,7 @@
         <v>2750</v>
       </c>
       <c r="C834" t="n">
-        <v>34272</v>
+        <v>40000</v>
       </c>
     </row>
     <row r="835">
@@ -9620,7 +9620,7 @@
         <v>1853</v>
       </c>
       <c r="C835" t="n">
-        <v>111420</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="836">
@@ -9631,7 +9631,7 @@
         <v>854</v>
       </c>
       <c r="C836" t="n">
-        <v>94284</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="837">
@@ -9642,7 +9642,7 @@
         <v>818</v>
       </c>
       <c r="C837" t="n">
-        <v>338562</v>
+        <v>395000</v>
       </c>
     </row>
     <row r="838">
@@ -9653,7 +9653,7 @@
         <v>2787</v>
       </c>
       <c r="C838" t="n">
-        <v>111428.59</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="839">
@@ -9664,7 +9664,7 @@
         <v>2684</v>
       </c>
       <c r="C839" t="n">
-        <v>83142</v>
+        <v>97000</v>
       </c>
     </row>
     <row r="840">
@@ -9675,7 +9675,7 @@
         <v>2653</v>
       </c>
       <c r="C840" t="n">
-        <v>102852</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="841">
@@ -9686,7 +9686,7 @@
         <v>2803</v>
       </c>
       <c r="C841" t="n">
-        <v>101988</v>
+        <v>119000</v>
       </c>
     </row>
     <row r="842">
@@ -9697,7 +9697,7 @@
         <v>2659</v>
       </c>
       <c r="C842" t="n">
-        <v>105444</v>
+        <v>123018.07</v>
       </c>
     </row>
     <row r="843">
@@ -9708,7 +9708,7 @@
         <v>2753</v>
       </c>
       <c r="C843" t="n">
-        <v>64278</v>
+        <v>75000</v>
       </c>
     </row>
     <row r="844">
@@ -9719,7 +9719,7 @@
         <v>2811</v>
       </c>
       <c r="C844" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="845">
@@ -9730,7 +9730,7 @@
         <v>2762</v>
       </c>
       <c r="C845" t="n">
-        <v>69840</v>
+        <v>81489.49000000001</v>
       </c>
     </row>
     <row r="846">
@@ -9741,7 +9741,7 @@
         <v>2702</v>
       </c>
       <c r="C846" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="847">
@@ -9752,7 +9752,7 @@
         <v>104</v>
       </c>
       <c r="C847" t="n">
-        <v>257130</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="848">
@@ -9763,7 +9763,7 @@
         <v>816</v>
       </c>
       <c r="C848" t="n">
-        <v>229590</v>
+        <v>267863</v>
       </c>
     </row>
     <row r="849">
@@ -9774,7 +9774,7 @@
         <v>1344</v>
       </c>
       <c r="C849" t="n">
-        <v>119988</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="850">
@@ -9785,7 +9785,7 @@
         <v>951</v>
       </c>
       <c r="C850" t="n">
-        <v>98568</v>
+        <v>115000</v>
       </c>
     </row>
     <row r="851">
@@ -9796,7 +9796,7 @@
         <v>2449</v>
       </c>
       <c r="C851" t="n">
-        <v>102852</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="852">
@@ -9807,7 +9807,7 @@
         <v>2709</v>
       </c>
       <c r="C852" t="n">
-        <v>154278</v>
+        <v>180000</v>
       </c>
     </row>
     <row r="853">
@@ -9840,7 +9840,7 @@
         <v>619</v>
       </c>
       <c r="C855" t="n">
-        <v>231930</v>
+        <v>270586.53</v>
       </c>
     </row>
     <row r="856">
@@ -9851,7 +9851,7 @@
         <v>2551</v>
       </c>
       <c r="C856" t="n">
-        <v>17550</v>
+        <v>20489.63</v>
       </c>
     </row>
     <row r="857">
@@ -9862,7 +9862,7 @@
         <v>2190</v>
       </c>
       <c r="C857" t="n">
-        <v>179136</v>
+        <v>209000</v>
       </c>
     </row>
     <row r="858">
@@ -9873,7 +9873,7 @@
         <v>2793</v>
       </c>
       <c r="C858" t="n">
-        <v>17142.86</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="859">
@@ -9884,7 +9884,7 @@
         <v>2687</v>
       </c>
       <c r="C859" t="n">
-        <v>85714.3</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="860">
@@ -9895,7 +9895,7 @@
         <v>2655</v>
       </c>
       <c r="C860" t="n">
-        <v>98568</v>
+        <v>115000</v>
       </c>
     </row>
     <row r="861">
@@ -9906,7 +9906,7 @@
         <v>2601</v>
       </c>
       <c r="C861" t="n">
-        <v>235710</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="862">
@@ -9917,7 +9917,7 @@
         <v>2745</v>
       </c>
       <c r="C862" t="n">
-        <v>94284</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="863">
@@ -9928,7 +9928,7 @@
         <v>794</v>
       </c>
       <c r="C863" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="864">
@@ -9939,7 +9939,7 @@
         <v>2586</v>
       </c>
       <c r="C864" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="865">
@@ -9950,7 +9950,7 @@
         <v>766</v>
       </c>
       <c r="C865" t="n">
-        <v>58878</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="866">
@@ -9961,7 +9961,7 @@
         <v>966</v>
       </c>
       <c r="C866" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="867">
@@ -9972,7 +9972,7 @@
         <v>749</v>
       </c>
       <c r="C867" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="868">
@@ -9983,7 +9983,7 @@
         <v>890</v>
       </c>
       <c r="C868" t="n">
-        <v>599994</v>
+        <v>700000</v>
       </c>
     </row>
     <row r="869">
@@ -9994,7 +9994,7 @@
         <v>2584</v>
       </c>
       <c r="C869" t="n">
-        <v>53946</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="870">
@@ -10005,7 +10005,7 @@
         <v>2363</v>
       </c>
       <c r="C870" t="n">
-        <v>124272</v>
+        <v>145000</v>
       </c>
     </row>
     <row r="871">
@@ -10016,7 +10016,7 @@
         <v>768</v>
       </c>
       <c r="C871" t="n">
-        <v>107136</v>
+        <v>125000</v>
       </c>
     </row>
     <row r="872">
@@ -10027,7 +10027,7 @@
         <v>2308</v>
       </c>
       <c r="C872" t="n">
-        <v>175698</v>
+        <v>205000</v>
       </c>
     </row>
     <row r="873">
@@ -10038,7 +10038,7 @@
         <v>1501</v>
       </c>
       <c r="C873" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="874">
@@ -10049,7 +10049,7 @@
         <v>675</v>
       </c>
       <c r="C874" t="n">
-        <v>171414</v>
+        <v>200000</v>
       </c>
     </row>
     <row r="875">
@@ -10060,7 +10060,7 @@
         <v>2783</v>
       </c>
       <c r="C875" t="n">
-        <v>60000.01</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="876">
@@ -10071,7 +10071,7 @@
         <v>2757</v>
       </c>
       <c r="C876" t="n">
-        <v>60000.01</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="877">
@@ -10082,7 +10082,7 @@
         <v>2266</v>
       </c>
       <c r="C877" t="n">
-        <v>68571.44</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="878">
@@ -10093,7 +10093,7 @@
         <v>351</v>
       </c>
       <c r="C878" t="n">
-        <v>162000</v>
+        <v>189000</v>
       </c>
     </row>
     <row r="879">
@@ -10104,7 +10104,7 @@
         <v>2383</v>
       </c>
       <c r="C879" t="n">
-        <v>120568.8</v>
+        <v>140667.9</v>
       </c>
     </row>
     <row r="880">
@@ -10115,7 +10115,7 @@
         <v>1585</v>
       </c>
       <c r="C880" t="n">
-        <v>141480</v>
+        <v>165061.84</v>
       </c>
     </row>
     <row r="881">
@@ -10126,7 +10126,7 @@
         <v>2330</v>
       </c>
       <c r="C881" t="n">
-        <v>231038.22</v>
+        <v>269550.93</v>
       </c>
     </row>
     <row r="882">
@@ -10137,7 +10137,7 @@
         <v>2413</v>
       </c>
       <c r="C882" t="n">
-        <v>103752</v>
+        <v>121045.35</v>
       </c>
     </row>
     <row r="883">
@@ -10148,7 +10148,7 @@
         <v>1450</v>
       </c>
       <c r="C883" t="n">
-        <v>233622</v>
+        <v>272574.37</v>
       </c>
     </row>
     <row r="884">
@@ -10159,7 +10159,7 @@
         <v>626</v>
       </c>
       <c r="C884" t="n">
-        <v>1460841.45</v>
+        <v>1704315</v>
       </c>
     </row>
     <row r="885">
@@ -10181,7 +10181,7 @@
         <v>89</v>
       </c>
       <c r="C886" t="n">
-        <v>289872</v>
+        <v>338186.71</v>
       </c>
     </row>
     <row r="887">
@@ -10192,7 +10192,7 @@
         <v>2146</v>
       </c>
       <c r="C887" t="n">
-        <v>172836</v>
+        <v>201656.31</v>
       </c>
     </row>
     <row r="888">
@@ -10203,7 +10203,7 @@
         <v>2223</v>
       </c>
       <c r="C888" t="n">
-        <v>113094</v>
+        <v>131947.96</v>
       </c>
     </row>
     <row r="889">
@@ -10214,7 +10214,7 @@
         <v>2633</v>
       </c>
       <c r="C889" t="n">
-        <v>14185.76</v>
+        <v>16550</v>
       </c>
     </row>
     <row r="890">
@@ -10225,7 +10225,7 @@
         <v>2577</v>
       </c>
       <c r="C890" t="n">
-        <v>76445.24000000001</v>
+        <v>89186.09</v>
       </c>
     </row>
     <row r="891">
@@ -10247,7 +10247,7 @@
         <v>559</v>
       </c>
       <c r="C892" t="n">
-        <v>214272</v>
+        <v>250000</v>
       </c>
     </row>
     <row r="893">
@@ -10258,7 +10258,7 @@
         <v>42</v>
       </c>
       <c r="C893" t="n">
-        <v>1635426</v>
+        <v>1908000</v>
       </c>
     </row>
     <row r="894">
@@ -10269,7 +10269,7 @@
         <v>663</v>
       </c>
       <c r="C894" t="n">
-        <v>228852</v>
+        <v>267000</v>
       </c>
     </row>
     <row r="895">
@@ -10291,7 +10291,7 @@
         <v>353</v>
       </c>
       <c r="C896" t="n">
-        <v>294814.96</v>
+        <v>343950.76</v>
       </c>
     </row>
     <row r="897">
@@ -10313,7 +10313,7 @@
         <v>2548</v>
       </c>
       <c r="C898" t="n">
-        <v>50148</v>
+        <v>58526.51</v>
       </c>
     </row>
     <row r="899">
@@ -10324,7 +10324,7 @@
         <v>2552</v>
       </c>
       <c r="C899" t="n">
-        <v>25344</v>
+        <v>29584.24</v>
       </c>
     </row>
     <row r="900">
@@ -10335,7 +10335,7 @@
         <v>1756</v>
       </c>
       <c r="C900" t="n">
-        <v>374148</v>
+        <v>436523.6</v>
       </c>
     </row>
     <row r="901">
@@ -10346,7 +10346,7 @@
         <v>2546</v>
       </c>
       <c r="C901" t="n">
-        <v>20448</v>
+        <v>23859.99</v>
       </c>
     </row>
     <row r="902">
@@ -10357,7 +10357,7 @@
         <v>2561</v>
       </c>
       <c r="C902" t="n">
-        <v>12600</v>
+        <v>14711.88</v>
       </c>
     </row>
     <row r="903">
@@ -10368,7 +10368,7 @@
         <v>415</v>
       </c>
       <c r="C903" t="n">
-        <v>453960</v>
+        <v>529635</v>
       </c>
     </row>
     <row r="904">
@@ -10379,7 +10379,7 @@
         <v>2727</v>
       </c>
       <c r="C904" t="n">
-        <v>38571.45</v>
+        <v>45000</v>
       </c>
     </row>
     <row r="905">
@@ -10390,7 +10390,7 @@
         <v>609</v>
       </c>
       <c r="C905" t="n">
-        <v>188571.43</v>
+        <v>220000</v>
       </c>
     </row>
     <row r="906">
@@ -10401,7 +10401,7 @@
         <v>1876</v>
       </c>
       <c r="C906" t="n">
-        <v>60000.01</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="907">
@@ -10412,7 +10412,7 @@
         <v>2718</v>
       </c>
       <c r="C907" t="n">
-        <v>59994</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="908">
@@ -10423,7 +10423,7 @@
         <v>2652</v>
       </c>
       <c r="C908" t="n">
-        <v>111420</v>
+        <v>130000</v>
       </c>
     </row>
     <row r="909">
@@ -10434,7 +10434,7 @@
         <v>2824</v>
       </c>
       <c r="C909" t="n">
-        <v>94285.73</v>
+        <v>110000</v>
       </c>
     </row>
     <row r="910">
@@ -10445,7 +10445,7 @@
         <v>952</v>
       </c>
       <c r="C910" t="n">
-        <v>77130</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="911">
@@ -10456,7 +10456,7 @@
         <v>1642</v>
       </c>
       <c r="C911" t="n">
-        <v>227142</v>
+        <v>265000</v>
       </c>
     </row>
     <row r="912">
@@ -10467,7 +10467,7 @@
         <v>744</v>
       </c>
       <c r="C912" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="913">
@@ -10478,7 +10478,7 @@
         <v>2323</v>
       </c>
       <c r="C913" t="n">
-        <v>58878</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="914">
@@ -10489,7 +10489,7 @@
         <v>970</v>
       </c>
       <c r="C914" t="n">
-        <v>58878</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="915">
@@ -10500,7 +10500,7 @@
         <v>2629</v>
       </c>
       <c r="C915" t="n">
-        <v>58878</v>
+        <v>68705.63</v>
       </c>
     </row>
     <row r="916">
@@ -10511,7 +10511,7 @@
         <v>933</v>
       </c>
       <c r="C916" t="n">
-        <v>69840</v>
+        <v>81489.46000000001</v>
       </c>
     </row>
     <row r="917">
@@ -10522,7 +10522,7 @@
         <v>2711</v>
       </c>
       <c r="C917" t="n">
-        <v>74322.8</v>
+        <v>86709.92</v>
       </c>
     </row>
     <row r="918">
@@ -10533,7 +10533,7 @@
         <v>1254</v>
       </c>
       <c r="C918" t="n">
-        <v>166457.17</v>
+        <v>194200</v>
       </c>
     </row>
     <row r="919">
@@ -10544,7 +10544,7 @@
         <v>2773</v>
       </c>
       <c r="C919" t="n">
-        <v>69171.45</v>
+        <v>80700</v>
       </c>
     </row>
     <row r="920">
@@ -10588,7 +10588,7 @@
         <v>530</v>
       </c>
       <c r="C923" t="n">
-        <v>209196</v>
+        <v>244071.88</v>
       </c>
     </row>
     <row r="924">
@@ -10599,7 +10599,7 @@
         <v>1810</v>
       </c>
       <c r="C924" t="n">
-        <v>30942</v>
+        <v>36104.13</v>
       </c>
     </row>
     <row r="925">
@@ -10610,7 +10610,7 @@
         <v>2045</v>
       </c>
       <c r="C925" t="n">
-        <v>288404.27</v>
+        <v>336471.62</v>
       </c>
     </row>
     <row r="926">
@@ -10632,7 +10632,7 @@
         <v>2755</v>
       </c>
       <c r="C927" t="n">
-        <v>51428.58</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="928">
@@ -10654,7 +10654,7 @@
         <v>2142</v>
       </c>
       <c r="C929" t="n">
-        <v>41220</v>
+        <v>48093.1</v>
       </c>
     </row>
     <row r="930">
@@ -10676,7 +10676,7 @@
         <v>2641</v>
       </c>
       <c r="C931" t="n">
-        <v>124272</v>
+        <v>145000</v>
       </c>
     </row>
     <row r="932">
@@ -10687,7 +10687,7 @@
         <v>1317</v>
       </c>
       <c r="C932" t="n">
-        <v>257130</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="933">
@@ -10720,7 +10720,7 @@
         <v>2463</v>
       </c>
       <c r="C935" t="n">
-        <v>265896</v>
+        <v>310224.87</v>
       </c>
     </row>
     <row r="936">
@@ -10731,7 +10731,7 @@
         <v>40</v>
       </c>
       <c r="C936" t="n">
-        <v>200844</v>
+        <v>234323.51</v>
       </c>
     </row>
     <row r="937">
@@ -10742,7 +10742,7 @@
         <v>1478</v>
       </c>
       <c r="C937" t="n">
-        <v>496980</v>
+        <v>579828.27</v>
       </c>
     </row>
     <row r="938">
@@ -10753,7 +10753,7 @@
         <v>2026</v>
       </c>
       <c r="C938" t="n">
-        <v>244275.25</v>
+        <v>284987.77</v>
       </c>
     </row>
     <row r="939">
@@ -10775,7 +10775,7 @@
         <v>2554</v>
       </c>
       <c r="C940" t="n">
-        <v>21042</v>
+        <v>24555.46</v>
       </c>
     </row>
     <row r="941">
@@ -10786,7 +10786,7 @@
         <v>1117</v>
       </c>
       <c r="C941" t="n">
-        <v>298188</v>
+        <v>347896.96</v>
       </c>
     </row>
     <row r="942">
@@ -10797,7 +10797,7 @@
         <v>2549</v>
       </c>
       <c r="C942" t="n">
-        <v>24300</v>
+        <v>28353.8</v>
       </c>
     </row>
     <row r="943">
@@ -10808,7 +10808,7 @@
         <v>2791</v>
       </c>
       <c r="C943" t="n">
-        <v>84600.03</v>
+        <v>98700</v>
       </c>
     </row>
     <row r="944">
@@ -10819,7 +10819,7 @@
         <v>2544</v>
       </c>
       <c r="C944" t="n">
-        <v>51426</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="945">
@@ -10830,7 +10830,7 @@
         <v>1492</v>
       </c>
       <c r="C945" t="n">
-        <v>68562</v>
+        <v>80000</v>
       </c>
     </row>
     <row r="946">
@@ -10841,7 +10841,7 @@
         <v>2131</v>
       </c>
       <c r="C946" t="n">
-        <v>119988</v>
+        <v>140000</v>
       </c>
     </row>
     <row r="947">
@@ -10852,7 +10852,7 @@
         <v>2663</v>
       </c>
       <c r="C947" t="n">
-        <v>235710</v>
+        <v>275000</v>
       </c>
     </row>
     <row r="948">
@@ -10863,7 +10863,7 @@
         <v>793</v>
       </c>
       <c r="C948" t="n">
-        <v>32094</v>
+        <v>37449.3</v>
       </c>
     </row>
     <row r="949">
@@ -10874,7 +10874,7 @@
         <v>2809</v>
       </c>
       <c r="C949" t="n">
-        <v>58878</v>
+        <v>68705.64999999999</v>
       </c>
     </row>
     <row r="950">
@@ -10885,7 +10885,7 @@
         <v>931</v>
       </c>
       <c r="C950" t="n">
-        <v>80928</v>
+        <v>94424.85000000001</v>
       </c>
     </row>
     <row r="951">
@@ -10896,7 +10896,7 @@
         <v>2345</v>
       </c>
       <c r="C951" t="n">
-        <v>53946</v>
+        <v>62949.9</v>
       </c>
     </row>
     <row r="952">
@@ -10907,7 +10907,7 @@
         <v>1381</v>
       </c>
       <c r="C952" t="n">
-        <v>252846</v>
+        <v>295000</v>
       </c>
     </row>
     <row r="953">
@@ -10918,7 +10918,7 @@
         <v>2124</v>
       </c>
       <c r="C953" t="n">
-        <v>282852</v>
+        <v>330000</v>
       </c>
     </row>
     <row r="954">
@@ -10929,7 +10929,7 @@
         <v>363</v>
       </c>
       <c r="C954" t="n">
-        <v>287136</v>
+        <v>335000</v>
       </c>
     </row>
     <row r="955">
@@ -10940,7 +10940,7 @@
         <v>703</v>
       </c>
       <c r="C955" t="n">
-        <v>197136</v>
+        <v>230000</v>
       </c>
     </row>
     <row r="956">
@@ -10951,7 +10951,7 @@
         <v>2748</v>
       </c>
       <c r="C956" t="n">
-        <v>60000.01</v>
+        <v>70000</v>
       </c>
     </row>
     <row r="957">
@@ -10962,7 +10962,7 @@
         <v>2673</v>
       </c>
       <c r="C957" t="n">
-        <v>85698</v>
+        <v>100000</v>
       </c>
     </row>
     <row r="958">
@@ -10973,7 +10973,7 @@
         <v>2118</v>
       </c>
       <c r="C958" t="n">
-        <v>202143.07</v>
+        <v>235839.18</v>
       </c>
     </row>
     <row r="959">
@@ -10984,7 +10984,7 @@
         <v>2325</v>
       </c>
       <c r="C959" t="n">
-        <v>136764</v>
+        <v>159559.78</v>
       </c>
     </row>
     <row r="960">
@@ -10995,7 +10995,7 @@
         <v>2678</v>
       </c>
       <c r="C960" t="n">
-        <v>291444.76</v>
+        <v>340027.38</v>
       </c>
     </row>
     <row r="961">
@@ -11006,7 +11006,7 @@
         <v>1906</v>
       </c>
       <c r="C961" t="n">
-        <v>97923.17</v>
+        <v>114244.3</v>
       </c>
     </row>
     <row r="962">
@@ -11017,7 +11017,7 @@
         <v>2607</v>
       </c>
       <c r="C962" t="n">
-        <v>42600.02</v>
+        <v>49700</v>
       </c>
     </row>
     <row r="963">
@@ -11028,7 +11028,7 @@
         <v>2251</v>
       </c>
       <c r="C963" t="n">
-        <v>183708</v>
+        <v>214342.76</v>
       </c>
     </row>
     <row r="964">
@@ -11039,7 +11039,7 @@
         <v>1116</v>
       </c>
       <c r="C964" t="n">
-        <v>217404</v>
+        <v>253640.38</v>
       </c>
     </row>
     <row r="965">
@@ -11050,7 +11050,7 @@
         <v>2651</v>
       </c>
       <c r="C965" t="n">
-        <v>144954</v>
+        <v>169120.47</v>
       </c>
     </row>
     <row r="966">
@@ -11061,7 +11061,7 @@
         <v>1063</v>
       </c>
       <c r="C966" t="n">
-        <v>311598</v>
+        <v>363550.99</v>
       </c>
     </row>
     <row r="967">
@@ -11072,7 +11072,7 @@
         <v>2580</v>
       </c>
       <c r="C967" t="n">
-        <v>28757.17</v>
+        <v>33550</v>
       </c>
     </row>
     <row r="968">
@@ -11094,7 +11094,7 @@
         <v>2141</v>
       </c>
       <c r="C969" t="n">
-        <v>24426</v>
+        <v>28507.85</v>
       </c>
     </row>
     <row r="970">
@@ -11116,7 +11116,7 @@
         <v>2660</v>
       </c>
       <c r="C971" t="n">
-        <v>257130</v>
+        <v>300000</v>
       </c>
     </row>
     <row r="972">
@@ -11138,7 +11138,7 @@
         <v>953</v>
       </c>
       <c r="C973" t="n">
-        <v>586854</v>
+        <v>684665.38</v>
       </c>
     </row>
     <row r="974">
@@ -11149,7 +11149,7 @@
         <v>483</v>
       </c>
       <c r="C974" t="n">
-        <v>379710</v>
+        <v>443000</v>
       </c>
     </row>
     <row r="975">
@@ -11160,7 +11160,7 @@
         <v>525</v>
       </c>
       <c r="C975" t="n">
-        <v>180000</v>
+        <v>210000</v>
       </c>
     </row>
     <row r="976">
@@ -11182,7 +11182,7 @@
         <v>424</v>
       </c>
       <c r="C977" t="n">
-        <v>198792</v>
+        <v>231931.31</v>
       </c>
     </row>
     <row r="978">
@@ -11204,7 +11204,7 @@
         <v>2550</v>
       </c>
       <c r="C979" t="n">
-        <v>52272</v>
+        <v>60987.41</v>
       </c>
     </row>
     <row r="980">
@@ -11215,7 +11215,7 @@
         <v>2555</v>
       </c>
       <c r="C980" t="n">
-        <v>35568</v>
+        <v>41514.24</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 07:37:30
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>2146</v>
       </c>
       <c r="C987" t="n">
-        <v>27498</v>
+        <v>54996</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>2325</v>
       </c>
       <c r="C988" t="n">
-        <v>21756</v>
+        <v>43512</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2547</v>
       </c>
       <c r="C989" t="n">
-        <v>5607</v>
+        <v>11214</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2552</v>
       </c>
       <c r="C990" t="n">
-        <v>4032</v>
+        <v>8064</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>949</v>
       </c>
       <c r="C991" t="n">
-        <v>13383</v>
+        <v>26766</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>2183</v>
       </c>
       <c r="C992" t="n">
-        <v>49902</v>
+        <v>99804</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>2394</v>
       </c>
       <c r="C993" t="n">
-        <v>21006</v>
+        <v>42012</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2413</v>
       </c>
       <c r="C994" t="n">
-        <v>16506</v>
+        <v>33012</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2341</v>
       </c>
       <c r="C995" t="n">
-        <v>19350</v>
+        <v>38700</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>1834</v>
       </c>
       <c r="C996" t="n">
-        <v>15954</v>
+        <v>31908</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2365</v>
       </c>
       <c r="C997" t="n">
-        <v>10863</v>
+        <v>21726</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2411</v>
       </c>
       <c r="C998" t="n">
-        <v>19350</v>
+        <v>38700</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2558</v>
       </c>
       <c r="C999" t="n">
-        <v>4098</v>
+        <v>8196</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2402</v>
       </c>
       <c r="C1000" t="n">
-        <v>88908</v>
+        <v>177816</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2085</v>
       </c>
       <c r="C1001" t="n">
-        <v>18006</v>
+        <v>36012</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>2568</v>
       </c>
       <c r="C1002" t="n">
-        <v>27876</v>
+        <v>55752</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>1871</v>
       </c>
       <c r="C1003" t="n">
-        <v>24102</v>
+        <v>48204</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2541</v>
       </c>
       <c r="C1004" t="n">
-        <v>28854</v>
+        <v>57708</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2647</v>
       </c>
       <c r="C1005" t="n">
-        <v>19350</v>
+        <v>38700</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>2562</v>
       </c>
       <c r="C1006" t="n">
-        <v>2157</v>
+        <v>4314</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>2567</v>
       </c>
       <c r="C1007" t="n">
-        <v>22506</v>
+        <v>45012</v>
       </c>
     </row>
     <row r="1008">
@@ -11523,7 +11523,7 @@
         <v>2510</v>
       </c>
       <c r="C1008" t="n">
-        <v>75714</v>
+        <v>151428</v>
       </c>
     </row>
     <row r="1009">
@@ -11534,7 +11534,7 @@
         <v>2392</v>
       </c>
       <c r="C1009" t="n">
-        <v>22713</v>
+        <v>45426</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>2613</v>
       </c>
       <c r="C1010" t="n">
-        <v>24435</v>
+        <v>48870</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2561</v>
       </c>
       <c r="C1011" t="n">
-        <v>2004</v>
+        <v>4008</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2643</v>
       </c>
       <c r="C1012" t="n">
-        <v>4026</v>
+        <v>8052</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>1456</v>
       </c>
       <c r="C1013" t="n">
-        <v>105039</v>
+        <v>210078</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2606</v>
       </c>
       <c r="C1014" t="n">
-        <v>32262</v>
+        <v>64524</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>1142</v>
       </c>
       <c r="C1015" t="n">
-        <v>58506</v>
+        <v>117012</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>1450</v>
       </c>
       <c r="C1016" t="n">
-        <v>37167</v>
+        <v>74334</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>2145</v>
       </c>
       <c r="C1017" t="n">
-        <v>17652</v>
+        <v>35304</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2574</v>
       </c>
       <c r="C1018" t="n">
-        <v>17652</v>
+        <v>35304</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>2492</v>
       </c>
       <c r="C1019" t="n">
-        <v>19350</v>
+        <v>38700</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2554</v>
       </c>
       <c r="C1020" t="n">
-        <v>3348</v>
+        <v>6696</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2556</v>
       </c>
       <c r="C1021" t="n">
-        <v>4923</v>
+        <v>9846</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>2546</v>
       </c>
       <c r="C1022" t="n">
-        <v>3252</v>
+        <v>6504</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2649</v>
       </c>
       <c r="C1023" t="n">
-        <v>4026</v>
+        <v>8052</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2082</v>
       </c>
       <c r="C1024" t="n">
-        <v>22713</v>
+        <v>45426</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>2223</v>
       </c>
       <c r="C1025" t="n">
-        <v>17991</v>
+        <v>35982</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2550</v>
       </c>
       <c r="C1026" t="n">
-        <v>8316</v>
+        <v>16632</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>2555</v>
       </c>
       <c r="C1027" t="n">
-        <v>5661</v>
+        <v>11322</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2627</v>
       </c>
       <c r="C1028" t="n">
-        <v>3324</v>
+        <v>6648</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2557</v>
       </c>
       <c r="C1029" t="n">
-        <v>3516</v>
+        <v>7032</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2551</v>
       </c>
       <c r="C1030" t="n">
-        <v>2793</v>
+        <v>5586</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>1907</v>
       </c>
       <c r="C1031" t="n">
-        <v>50589</v>
+        <v>101178</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>2705</v>
       </c>
       <c r="C1032" t="n">
-        <v>24435</v>
+        <v>48870</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2333</v>
       </c>
       <c r="C1033" t="n">
-        <v>21048</v>
+        <v>42096</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2548</v>
       </c>
       <c r="C1034" t="n">
-        <v>7980</v>
+        <v>15960</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2549</v>
       </c>
       <c r="C1035" t="n">
-        <v>3864</v>
+        <v>7728</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2249</v>
       </c>
       <c r="C1036" t="n">
-        <v>26634</v>
+        <v>53268</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>1585</v>
       </c>
       <c r="C1037" t="n">
-        <v>22506</v>
+        <v>45012</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2276</v>
       </c>
       <c r="C1038" t="n">
-        <v>30552</v>
+        <v>61104</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
chore(data): batch update intraday meta_faturamento - 08:00:54
</commit_message>
<xml_diff>
--- a/data/meta_faturamento.xlsx
+++ b/data/meta_faturamento.xlsx
@@ -11292,7 +11292,7 @@
         <v>2146</v>
       </c>
       <c r="C987" t="n">
-        <v>54996</v>
+        <v>64162</v>
       </c>
     </row>
     <row r="988">
@@ -11303,7 +11303,7 @@
         <v>2325</v>
       </c>
       <c r="C988" t="n">
-        <v>43512</v>
+        <v>50764</v>
       </c>
     </row>
     <row r="989">
@@ -11314,7 +11314,7 @@
         <v>2547</v>
       </c>
       <c r="C989" t="n">
-        <v>11214</v>
+        <v>13083</v>
       </c>
     </row>
     <row r="990">
@@ -11325,7 +11325,7 @@
         <v>2552</v>
       </c>
       <c r="C990" t="n">
-        <v>8064</v>
+        <v>9408</v>
       </c>
     </row>
     <row r="991">
@@ -11336,7 +11336,7 @@
         <v>949</v>
       </c>
       <c r="C991" t="n">
-        <v>26766</v>
+        <v>31227</v>
       </c>
     </row>
     <row r="992">
@@ -11347,7 +11347,7 @@
         <v>2183</v>
       </c>
       <c r="C992" t="n">
-        <v>99804</v>
+        <v>116438</v>
       </c>
     </row>
     <row r="993">
@@ -11358,7 +11358,7 @@
         <v>2394</v>
       </c>
       <c r="C993" t="n">
-        <v>42012</v>
+        <v>49014</v>
       </c>
     </row>
     <row r="994">
@@ -11369,7 +11369,7 @@
         <v>2413</v>
       </c>
       <c r="C994" t="n">
-        <v>33012</v>
+        <v>38514</v>
       </c>
     </row>
     <row r="995">
@@ -11380,7 +11380,7 @@
         <v>2341</v>
       </c>
       <c r="C995" t="n">
-        <v>38700</v>
+        <v>45150</v>
       </c>
     </row>
     <row r="996">
@@ -11391,7 +11391,7 @@
         <v>1834</v>
       </c>
       <c r="C996" t="n">
-        <v>31908</v>
+        <v>37226</v>
       </c>
     </row>
     <row r="997">
@@ -11402,7 +11402,7 @@
         <v>2365</v>
       </c>
       <c r="C997" t="n">
-        <v>21726</v>
+        <v>25347</v>
       </c>
     </row>
     <row r="998">
@@ -11413,7 +11413,7 @@
         <v>2411</v>
       </c>
       <c r="C998" t="n">
-        <v>38700</v>
+        <v>45150</v>
       </c>
     </row>
     <row r="999">
@@ -11424,7 +11424,7 @@
         <v>2558</v>
       </c>
       <c r="C999" t="n">
-        <v>8196</v>
+        <v>9562</v>
       </c>
     </row>
     <row r="1000">
@@ -11435,7 +11435,7 @@
         <v>2402</v>
       </c>
       <c r="C1000" t="n">
-        <v>177816</v>
+        <v>207452</v>
       </c>
     </row>
     <row r="1001">
@@ -11446,7 +11446,7 @@
         <v>2085</v>
       </c>
       <c r="C1001" t="n">
-        <v>36012</v>
+        <v>42014</v>
       </c>
     </row>
     <row r="1002">
@@ -11457,7 +11457,7 @@
         <v>2568</v>
       </c>
       <c r="C1002" t="n">
-        <v>55752</v>
+        <v>65044</v>
       </c>
     </row>
     <row r="1003">
@@ -11468,7 +11468,7 @@
         <v>1871</v>
       </c>
       <c r="C1003" t="n">
-        <v>48204</v>
+        <v>56238</v>
       </c>
     </row>
     <row r="1004">
@@ -11479,7 +11479,7 @@
         <v>2541</v>
       </c>
       <c r="C1004" t="n">
-        <v>57708</v>
+        <v>67326</v>
       </c>
     </row>
     <row r="1005">
@@ -11490,7 +11490,7 @@
         <v>2647</v>
       </c>
       <c r="C1005" t="n">
-        <v>38700</v>
+        <v>45150</v>
       </c>
     </row>
     <row r="1006">
@@ -11501,7 +11501,7 @@
         <v>2562</v>
       </c>
       <c r="C1006" t="n">
-        <v>4314</v>
+        <v>5033</v>
       </c>
     </row>
     <row r="1007">
@@ -11512,7 +11512,7 @@
         <v>2567</v>
       </c>
       <c r="C1007" t="n">
-        <v>45012</v>
+        <v>52514</v>
       </c>
     </row>
     <row r="1008">
@@ -11523,7 +11523,7 @@
         <v>2510</v>
       </c>
       <c r="C1008" t="n">
-        <v>151428</v>
+        <v>176666</v>
       </c>
     </row>
     <row r="1009">
@@ -11534,7 +11534,7 @@
         <v>2392</v>
       </c>
       <c r="C1009" t="n">
-        <v>45426</v>
+        <v>52997</v>
       </c>
     </row>
     <row r="1010">
@@ -11545,7 +11545,7 @@
         <v>2613</v>
       </c>
       <c r="C1010" t="n">
-        <v>48870</v>
+        <v>57015</v>
       </c>
     </row>
     <row r="1011">
@@ -11556,7 +11556,7 @@
         <v>2561</v>
       </c>
       <c r="C1011" t="n">
-        <v>4008</v>
+        <v>4676</v>
       </c>
     </row>
     <row r="1012">
@@ -11567,7 +11567,7 @@
         <v>2643</v>
       </c>
       <c r="C1012" t="n">
-        <v>8052</v>
+        <v>9394</v>
       </c>
     </row>
     <row r="1013">
@@ -11578,7 +11578,7 @@
         <v>1456</v>
       </c>
       <c r="C1013" t="n">
-        <v>210078</v>
+        <v>245091</v>
       </c>
     </row>
     <row r="1014">
@@ -11589,7 +11589,7 @@
         <v>2606</v>
       </c>
       <c r="C1014" t="n">
-        <v>64524</v>
+        <v>75278</v>
       </c>
     </row>
     <row r="1015">
@@ -11600,7 +11600,7 @@
         <v>1142</v>
       </c>
       <c r="C1015" t="n">
-        <v>117012</v>
+        <v>136514</v>
       </c>
     </row>
     <row r="1016">
@@ -11611,7 +11611,7 @@
         <v>1450</v>
       </c>
       <c r="C1016" t="n">
-        <v>74334</v>
+        <v>86723</v>
       </c>
     </row>
     <row r="1017">
@@ -11622,7 +11622,7 @@
         <v>2145</v>
       </c>
       <c r="C1017" t="n">
-        <v>35304</v>
+        <v>41188</v>
       </c>
     </row>
     <row r="1018">
@@ -11633,7 +11633,7 @@
         <v>2574</v>
       </c>
       <c r="C1018" t="n">
-        <v>35304</v>
+        <v>41188</v>
       </c>
     </row>
     <row r="1019">
@@ -11644,7 +11644,7 @@
         <v>2492</v>
       </c>
       <c r="C1019" t="n">
-        <v>38700</v>
+        <v>45150</v>
       </c>
     </row>
     <row r="1020">
@@ -11655,7 +11655,7 @@
         <v>2554</v>
       </c>
       <c r="C1020" t="n">
-        <v>6696</v>
+        <v>7812</v>
       </c>
     </row>
     <row r="1021">
@@ -11666,7 +11666,7 @@
         <v>2556</v>
       </c>
       <c r="C1021" t="n">
-        <v>9846</v>
+        <v>11487</v>
       </c>
     </row>
     <row r="1022">
@@ -11677,7 +11677,7 @@
         <v>2546</v>
       </c>
       <c r="C1022" t="n">
-        <v>6504</v>
+        <v>7588</v>
       </c>
     </row>
     <row r="1023">
@@ -11688,7 +11688,7 @@
         <v>2649</v>
       </c>
       <c r="C1023" t="n">
-        <v>8052</v>
+        <v>9394</v>
       </c>
     </row>
     <row r="1024">
@@ -11699,7 +11699,7 @@
         <v>2082</v>
       </c>
       <c r="C1024" t="n">
-        <v>45426</v>
+        <v>52997</v>
       </c>
     </row>
     <row r="1025">
@@ -11710,7 +11710,7 @@
         <v>2223</v>
       </c>
       <c r="C1025" t="n">
-        <v>35982</v>
+        <v>41979</v>
       </c>
     </row>
     <row r="1026">
@@ -11721,7 +11721,7 @@
         <v>2550</v>
       </c>
       <c r="C1026" t="n">
-        <v>16632</v>
+        <v>19404</v>
       </c>
     </row>
     <row r="1027">
@@ -11732,7 +11732,7 @@
         <v>2555</v>
       </c>
       <c r="C1027" t="n">
-        <v>11322</v>
+        <v>13209</v>
       </c>
     </row>
     <row r="1028">
@@ -11743,7 +11743,7 @@
         <v>2627</v>
       </c>
       <c r="C1028" t="n">
-        <v>6648</v>
+        <v>7756</v>
       </c>
     </row>
     <row r="1029">
@@ -11754,7 +11754,7 @@
         <v>2557</v>
       </c>
       <c r="C1029" t="n">
-        <v>7032</v>
+        <v>8204</v>
       </c>
     </row>
     <row r="1030">
@@ -11765,7 +11765,7 @@
         <v>2551</v>
       </c>
       <c r="C1030" t="n">
-        <v>5586</v>
+        <v>6517</v>
       </c>
     </row>
     <row r="1031">
@@ -11776,7 +11776,7 @@
         <v>1907</v>
       </c>
       <c r="C1031" t="n">
-        <v>101178</v>
+        <v>118041</v>
       </c>
     </row>
     <row r="1032">
@@ -11787,7 +11787,7 @@
         <v>2705</v>
       </c>
       <c r="C1032" t="n">
-        <v>48870</v>
+        <v>57015</v>
       </c>
     </row>
     <row r="1033">
@@ -11798,7 +11798,7 @@
         <v>2333</v>
       </c>
       <c r="C1033" t="n">
-        <v>42096</v>
+        <v>49112</v>
       </c>
     </row>
     <row r="1034">
@@ -11809,7 +11809,7 @@
         <v>2548</v>
       </c>
       <c r="C1034" t="n">
-        <v>15960</v>
+        <v>18620</v>
       </c>
     </row>
     <row r="1035">
@@ -11820,7 +11820,7 @@
         <v>2549</v>
       </c>
       <c r="C1035" t="n">
-        <v>7728</v>
+        <v>9016</v>
       </c>
     </row>
     <row r="1036">
@@ -11831,7 +11831,7 @@
         <v>2249</v>
       </c>
       <c r="C1036" t="n">
-        <v>53268</v>
+        <v>62146</v>
       </c>
     </row>
     <row r="1037">
@@ -11842,7 +11842,7 @@
         <v>1585</v>
       </c>
       <c r="C1037" t="n">
-        <v>45012</v>
+        <v>52514</v>
       </c>
     </row>
     <row r="1038">
@@ -11853,7 +11853,7 @@
         <v>2276</v>
       </c>
       <c r="C1038" t="n">
-        <v>61104</v>
+        <v>71288</v>
       </c>
     </row>
   </sheetData>

</xml_diff>